<commit_message>
fix(brand): 🩹 Sync ai4comms charter — overlay, logo-on-image, palette
Charter alignment from client-data 0d3c8fb: canopy-green image overlay
per guidelines, logo-on-image resolves to the real (only) variant,
primary table headers, diversified chart palette.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client-data/clients/ai4comms/ai4comms-client-data-overview.xlsx
+++ b/client-data/clients/ai4comms/ai4comms-client-data-overview.xlsx
@@ -730,7 +730,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>174</t>
         </is>
       </c>
     </row>
@@ -778,7 +778,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -790,7 +790,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -820,7 +820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F179"/>
+  <dimension ref="A1:F196"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1314,22 +1314,22 @@
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>assets/svg/divider-full.svg</t>
+          <t>ai4comms-client-data-overview.xlsx</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>assets</t>
+          <t>root</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>SVG</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>0.8 KB</t>
+          <t>17.5 KB</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
@@ -1341,7 +1341,7 @@
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>assets/svg/divider-minimal.svg</t>
+          <t>assets/svg/divider-full.svg</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
@@ -1356,7 +1356,7 @@
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>0.2 KB</t>
+          <t>0.8 KB</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
@@ -1368,7 +1368,7 @@
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>assets/svg/divider-short.svg</t>
+          <t>assets/svg/divider-minimal.svg</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>0.3 KB</t>
+          <t>0.2 KB</t>
         </is>
       </c>
       <c r="E23" s="10" t="inlineStr">
@@ -1395,7 +1395,7 @@
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>assets/svg/pattern-tile.svg</t>
+          <t>assets/svg/divider-short.svg</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
@@ -1410,7 +1410,7 @@
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>0.5 KB</t>
+          <t>0.3 KB</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr">
@@ -1422,39 +1422,39 @@
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>charter.json</t>
+          <t>assets/svg/pattern-tile.svg</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>root</t>
+          <t>assets</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>JSON</t>
+          <t>SVG</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>7.9 KB</t>
+          <t>0.5 KB</t>
         </is>
       </c>
       <c r="E25" s="10" t="inlineStr">
         <is>
-          <t>Brand identity spec — colors, typography, logos, images, templates</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>guidelines.md</t>
+          <t>business-cards/print/README.md</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>root</t>
+          <t>business-cards</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
@@ -1464,505 +1464,505 @@
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>8.5 KB</t>
+          <t>2.0 KB</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>Brand usage guidelines</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-03-AMWQIpdsSHY--16x9-textsafe.jpg</t>
+          <t>business-cards/print/arien-eu-print.pdf</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>business-cards</t>
         </is>
       </c>
       <c r="C27" s="9" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>PDF</t>
         </is>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>73.8 KB</t>
+          <t>69.3 KB</t>
         </is>
       </c>
       <c r="E27" s="10" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-03-AMWQIpdsSHY--16x9.jpg</t>
+          <t>business-cards/print/emma-eu-print.pdf</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>business-cards</t>
         </is>
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>PDF</t>
         </is>
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>101.2 KB</t>
+          <t>70.0 KB</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-03-AMWQIpdsSHY--1x1-textsafe.jpg</t>
+          <t>business-cards/print/ingo-eu-print.pdf</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>business-cards</t>
         </is>
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>PDF</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>51.5 KB</t>
+          <t>69.9 KB</t>
         </is>
       </c>
       <c r="E29" s="10" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-03-AMWQIpdsSHY--1x1.jpg</t>
+          <t>business-cards/print/william-eu-print.pdf</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>business-cards</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>PDF</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>71.5 KB</t>
+          <t>71.2 KB</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-03-AMWQIpdsSHY--2x1-textsafe.jpg</t>
+          <t>business-cards/review/business-cards.html</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>business-cards</t>
         </is>
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>HTML</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>64.7 KB</t>
+          <t>3.7 KB</t>
         </is>
       </c>
       <c r="E31" s="10" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-03-AMWQIpdsSHY--2x1.jpg</t>
+          <t>business-cards/source/arien-eu-front.svg</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>business-cards</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>SVG</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>88.6 KB</t>
+          <t>1.6 KB</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-03-AMWQIpdsSHY.jpg</t>
+          <t>business-cards/source/back-eu.svg</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>business-cards</t>
         </is>
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>SVG</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>137.1 KB</t>
+          <t>1.4 KB</t>
         </is>
       </c>
       <c r="E33" s="10" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-04-cd7i9vYIyeY--16x9-textsafe.jpg</t>
+          <t>business-cards/source/emma-eu-front.svg</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>business-cards</t>
         </is>
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>SVG</t>
         </is>
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>69.8 KB</t>
+          <t>1.6 KB</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-04-cd7i9vYIyeY--16x9.jpg</t>
+          <t>business-cards/source/ingo-eu-front.svg</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>business-cards</t>
         </is>
       </c>
       <c r="C35" s="9" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>SVG</t>
         </is>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>95.9 KB</t>
+          <t>1.6 KB</t>
         </is>
       </c>
       <c r="E35" s="10" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="36" ht="16" customHeight="1">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-04-cd7i9vYIyeY--1x1-textsafe.jpg</t>
+          <t>business-cards/source/william-eu-front.svg</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>business-cards</t>
         </is>
       </c>
       <c r="C36" s="11" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>SVG</t>
         </is>
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>52.6 KB</t>
+          <t>1.6 KB</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-04-cd7i9vYIyeY--1x1.jpg</t>
+          <t>charter.json</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>root</t>
         </is>
       </c>
       <c r="C37" s="9" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>JSON</t>
         </is>
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>71.7 KB</t>
+          <t>8.2 KB</t>
         </is>
       </c>
       <c r="E37" s="10" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>Brand identity spec — colors, typography, logos, images, templates</t>
         </is>
       </c>
     </row>
     <row r="38" ht="16" customHeight="1">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-04-cd7i9vYIyeY--2x1-textsafe.jpg</t>
+          <t>fonts/JetBrainsMono-Bold.ttf</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>fonts</t>
         </is>
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>Font TTF</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>65.7 KB</t>
+          <t>112.1 KB</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>Font file — JetBrainsMono-Bold</t>
         </is>
       </c>
     </row>
     <row r="39" ht="16" customHeight="1">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-04-cd7i9vYIyeY--2x1.jpg</t>
+          <t>fonts/JetBrainsMono-OFL.txt</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>fonts</t>
         </is>
       </c>
       <c r="C39" s="9" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>89.6 KB</t>
+          <t>4.3 KB</t>
         </is>
       </c>
       <c r="E39" s="10" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>Font file — JetBrainsMono-OFL</t>
         </is>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1">
       <c r="A40" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-04-cd7i9vYIyeY.jpg</t>
+          <t>fonts/JetBrainsMono-Regular.ttf</t>
         </is>
       </c>
       <c r="B40" s="11" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>fonts</t>
         </is>
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>Font TTF</t>
         </is>
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>132.9 KB</t>
+          <t>112.2 KB</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>Font file — JetBrainsMono-Regular</t>
         </is>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-05-u36g8i9nCao--16x9-textsafe.jpg</t>
+          <t>fonts/Montserrat-Italic[wght].ttf</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>fonts</t>
         </is>
       </c>
       <c r="C41" s="9" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>Font TTF</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>105.8 KB</t>
+          <t>744.5 KB</t>
         </is>
       </c>
       <c r="E41" s="10" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>Font file — Montserrat-Italic[wght]</t>
         </is>
       </c>
     </row>
     <row r="42" ht="16" customHeight="1">
       <c r="A42" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-05-u36g8i9nCao--16x9.jpg</t>
+          <t>fonts/Montserrat[wght].ttf</t>
         </is>
       </c>
       <c r="B42" s="11" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>fonts</t>
         </is>
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>Font TTF</t>
         </is>
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>148.8 KB</t>
+          <t>727.5 KB</t>
         </is>
       </c>
       <c r="E42" s="12" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>Font file — Montserrat[wght]</t>
         </is>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-05-u36g8i9nCao--1x1-textsafe.jpg</t>
+          <t>fonts/OFL-Montserrat.txt</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>fonts</t>
         </is>
       </c>
       <c r="C43" s="9" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>98.1 KB</t>
+          <t>4.3 KB</t>
         </is>
       </c>
       <c r="E43" s="10" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>Font file — OFL-Montserrat</t>
         </is>
       </c>
     </row>
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-05-u36g8i9nCao--1x1.jpg</t>
+          <t>guidelines.md</t>
         </is>
       </c>
       <c r="B44" s="11" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>root</t>
         </is>
       </c>
       <c r="C44" s="11" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>Markdown</t>
         </is>
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>132.6 KB</t>
+          <t>8.5 KB</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>Brand usage guidelines</t>
         </is>
       </c>
     </row>
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-05-u36g8i9nCao--2x1-textsafe.jpg</t>
+          <t>images/comms-env-03-AMWQIpdsSHY--16x9-textsafe.jpg</t>
         </is>
       </c>
       <c r="B45" s="9" t="inlineStr">
@@ -1977,7 +1977,7 @@
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>97.6 KB</t>
+          <t>73.8 KB</t>
         </is>
       </c>
       <c r="E45" s="10" t="inlineStr">
@@ -1989,7 +1989,7 @@
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-05-u36g8i9nCao--2x1.jpg</t>
+          <t>images/comms-env-03-AMWQIpdsSHY--16x9.jpg</t>
         </is>
       </c>
       <c r="B46" s="11" t="inlineStr">
@@ -2004,7 +2004,7 @@
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>136.7 KB</t>
+          <t>101.2 KB</t>
         </is>
       </c>
       <c r="E46" s="12" t="inlineStr">
@@ -2016,7 +2016,7 @@
     <row r="47" ht="16" customHeight="1">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-05-u36g8i9nCao.jpg</t>
+          <t>images/comms-env-03-AMWQIpdsSHY--1x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B47" s="9" t="inlineStr">
@@ -2031,7 +2031,7 @@
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>176.9 KB</t>
+          <t>51.5 KB</t>
         </is>
       </c>
       <c r="E47" s="10" t="inlineStr">
@@ -2043,7 +2043,7 @@
     <row r="48" ht="16" customHeight="1">
       <c r="A48" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-06-GP7SH7RRkqo--16x9-textsafe.jpg</t>
+          <t>images/comms-env-03-AMWQIpdsSHY--1x1.jpg</t>
         </is>
       </c>
       <c r="B48" s="11" t="inlineStr">
@@ -2058,7 +2058,7 @@
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>215.1 KB</t>
+          <t>71.5 KB</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
@@ -2070,7 +2070,7 @@
     <row r="49" ht="16" customHeight="1">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-06-GP7SH7RRkqo--16x9.jpg</t>
+          <t>images/comms-env-03-AMWQIpdsSHY--2x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B49" s="9" t="inlineStr">
@@ -2085,7 +2085,7 @@
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>286.1 KB</t>
+          <t>64.7 KB</t>
         </is>
       </c>
       <c r="E49" s="10" t="inlineStr">
@@ -2097,7 +2097,7 @@
     <row r="50" ht="16" customHeight="1">
       <c r="A50" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-06-GP7SH7RRkqo--1x1-textsafe.jpg</t>
+          <t>images/comms-env-03-AMWQIpdsSHY--2x1.jpg</t>
         </is>
       </c>
       <c r="B50" s="11" t="inlineStr">
@@ -2112,7 +2112,7 @@
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>137.4 KB</t>
+          <t>88.6 KB</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr">
@@ -2124,7 +2124,7 @@
     <row r="51" ht="16" customHeight="1">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-06-GP7SH7RRkqo--1x1.jpg</t>
+          <t>images/comms-env-03-AMWQIpdsSHY.jpg</t>
         </is>
       </c>
       <c r="B51" s="9" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>184.0 KB</t>
+          <t>137.1 KB</t>
         </is>
       </c>
       <c r="E51" s="10" t="inlineStr">
@@ -2151,7 +2151,7 @@
     <row r="52" ht="16" customHeight="1">
       <c r="A52" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-06-GP7SH7RRkqo--2x1-textsafe.jpg</t>
+          <t>images/comms-env-04-cd7i9vYIyeY--16x9-textsafe.jpg</t>
         </is>
       </c>
       <c r="B52" s="11" t="inlineStr">
@@ -2166,7 +2166,7 @@
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>196.6 KB</t>
+          <t>69.8 KB</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
@@ -2178,7 +2178,7 @@
     <row r="53" ht="16" customHeight="1">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-06-GP7SH7RRkqo--2x1.jpg</t>
+          <t>images/comms-env-04-cd7i9vYIyeY--16x9.jpg</t>
         </is>
       </c>
       <c r="B53" s="9" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>260.4 KB</t>
+          <t>95.9 KB</t>
         </is>
       </c>
       <c r="E53" s="10" t="inlineStr">
@@ -2205,7 +2205,7 @@
     <row r="54" ht="16" customHeight="1">
       <c r="A54" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-06-GP7SH7RRkqo.jpg</t>
+          <t>images/comms-env-04-cd7i9vYIyeY--1x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B54" s="11" t="inlineStr">
@@ -2220,7 +2220,7 @@
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>365.4 KB</t>
+          <t>52.6 KB</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
@@ -2232,7 +2232,7 @@
     <row r="55" ht="16" customHeight="1">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-07-qoJpt9Ja6y0--16x9-textsafe.jpg</t>
+          <t>images/comms-env-04-cd7i9vYIyeY--1x1.jpg</t>
         </is>
       </c>
       <c r="B55" s="9" t="inlineStr">
@@ -2247,7 +2247,7 @@
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>23.5 KB</t>
+          <t>71.7 KB</t>
         </is>
       </c>
       <c r="E55" s="10" t="inlineStr">
@@ -2259,7 +2259,7 @@
     <row r="56" ht="16" customHeight="1">
       <c r="A56" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-07-qoJpt9Ja6y0--16x9.jpg</t>
+          <t>images/comms-env-04-cd7i9vYIyeY--2x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B56" s="11" t="inlineStr">
@@ -2274,7 +2274,7 @@
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>32.9 KB</t>
+          <t>65.7 KB</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
@@ -2286,7 +2286,7 @@
     <row r="57" ht="16" customHeight="1">
       <c r="A57" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-07-qoJpt9Ja6y0--1x1-textsafe.jpg</t>
+          <t>images/comms-env-04-cd7i9vYIyeY--2x1.jpg</t>
         </is>
       </c>
       <c r="B57" s="9" t="inlineStr">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>17.9 KB</t>
+          <t>89.6 KB</t>
         </is>
       </c>
       <c r="E57" s="10" t="inlineStr">
@@ -2313,7 +2313,7 @@
     <row r="58" ht="16" customHeight="1">
       <c r="A58" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-07-qoJpt9Ja6y0--1x1.jpg</t>
+          <t>images/comms-env-04-cd7i9vYIyeY.jpg</t>
         </is>
       </c>
       <c r="B58" s="11" t="inlineStr">
@@ -2328,7 +2328,7 @@
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>25.5 KB</t>
+          <t>132.9 KB</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
@@ -2340,7 +2340,7 @@
     <row r="59" ht="16" customHeight="1">
       <c r="A59" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-07-qoJpt9Ja6y0--2x1-textsafe.jpg</t>
+          <t>images/comms-env-05-u36g8i9nCao--16x9-textsafe.jpg</t>
         </is>
       </c>
       <c r="B59" s="9" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>22.0 KB</t>
+          <t>105.8 KB</t>
         </is>
       </c>
       <c r="E59" s="10" t="inlineStr">
@@ -2367,7 +2367,7 @@
     <row r="60" ht="16" customHeight="1">
       <c r="A60" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-07-qoJpt9Ja6y0--2x1.jpg</t>
+          <t>images/comms-env-05-u36g8i9nCao--16x9.jpg</t>
         </is>
       </c>
       <c r="B60" s="11" t="inlineStr">
@@ -2382,7 +2382,7 @@
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>30.7 KB</t>
+          <t>148.8 KB</t>
         </is>
       </c>
       <c r="E60" s="12" t="inlineStr">
@@ -2394,7 +2394,7 @@
     <row r="61" ht="16" customHeight="1">
       <c r="A61" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-07-qoJpt9Ja6y0.jpg</t>
+          <t>images/comms-env-05-u36g8i9nCao--1x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B61" s="9" t="inlineStr">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>40.9 KB</t>
+          <t>98.1 KB</t>
         </is>
       </c>
       <c r="E61" s="10" t="inlineStr">
@@ -2421,7 +2421,7 @@
     <row r="62" ht="16" customHeight="1">
       <c r="A62" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-08-bGo01h57aCE--16x9-textsafe.jpg</t>
+          <t>images/comms-env-05-u36g8i9nCao--1x1.jpg</t>
         </is>
       </c>
       <c r="B62" s="11" t="inlineStr">
@@ -2436,7 +2436,7 @@
       </c>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>84.0 KB</t>
+          <t>132.6 KB</t>
         </is>
       </c>
       <c r="E62" s="12" t="inlineStr">
@@ -2448,7 +2448,7 @@
     <row r="63" ht="16" customHeight="1">
       <c r="A63" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-08-bGo01h57aCE--16x9.jpg</t>
+          <t>images/comms-env-05-u36g8i9nCao--2x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B63" s="9" t="inlineStr">
@@ -2463,7 +2463,7 @@
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>105.3 KB</t>
+          <t>97.6 KB</t>
         </is>
       </c>
       <c r="E63" s="10" t="inlineStr">
@@ -2475,7 +2475,7 @@
     <row r="64" ht="16" customHeight="1">
       <c r="A64" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-08-bGo01h57aCE--1x1-textsafe.jpg</t>
+          <t>images/comms-env-05-u36g8i9nCao--2x1.jpg</t>
         </is>
       </c>
       <c r="B64" s="11" t="inlineStr">
@@ -2490,7 +2490,7 @@
       </c>
       <c r="D64" s="11" t="inlineStr">
         <is>
-          <t>61.0 KB</t>
+          <t>136.7 KB</t>
         </is>
       </c>
       <c r="E64" s="12" t="inlineStr">
@@ -2502,7 +2502,7 @@
     <row r="65" ht="16" customHeight="1">
       <c r="A65" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-08-bGo01h57aCE--1x1.jpg</t>
+          <t>images/comms-env-05-u36g8i9nCao.jpg</t>
         </is>
       </c>
       <c r="B65" s="9" t="inlineStr">
@@ -2517,7 +2517,7 @@
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>75.6 KB</t>
+          <t>176.9 KB</t>
         </is>
       </c>
       <c r="E65" s="10" t="inlineStr">
@@ -2529,7 +2529,7 @@
     <row r="66" ht="16" customHeight="1">
       <c r="A66" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-08-bGo01h57aCE--2x1-textsafe.jpg</t>
+          <t>images/comms-env-06-GP7SH7RRkqo--16x9-textsafe.jpg</t>
         </is>
       </c>
       <c r="B66" s="11" t="inlineStr">
@@ -2544,7 +2544,7 @@
       </c>
       <c r="D66" s="11" t="inlineStr">
         <is>
-          <t>82.0 KB</t>
+          <t>215.1 KB</t>
         </is>
       </c>
       <c r="E66" s="12" t="inlineStr">
@@ -2556,7 +2556,7 @@
     <row r="67" ht="16" customHeight="1">
       <c r="A67" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-08-bGo01h57aCE--2x1.jpg</t>
+          <t>images/comms-env-06-GP7SH7RRkqo--16x9.jpg</t>
         </is>
       </c>
       <c r="B67" s="9" t="inlineStr">
@@ -2571,7 +2571,7 @@
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>101.9 KB</t>
+          <t>286.1 KB</t>
         </is>
       </c>
       <c r="E67" s="10" t="inlineStr">
@@ -2583,7 +2583,7 @@
     <row r="68" ht="16" customHeight="1">
       <c r="A68" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-08-bGo01h57aCE.jpg</t>
+          <t>images/comms-env-06-GP7SH7RRkqo--1x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B68" s="11" t="inlineStr">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="D68" s="11" t="inlineStr">
         <is>
-          <t>118.8 KB</t>
+          <t>137.4 KB</t>
         </is>
       </c>
       <c r="E68" s="12" t="inlineStr">
@@ -2610,7 +2610,7 @@
     <row r="69" ht="16" customHeight="1">
       <c r="A69" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-09-_Y-32yPvO0k--16x9-textsafe.jpg</t>
+          <t>images/comms-env-06-GP7SH7RRkqo--1x1.jpg</t>
         </is>
       </c>
       <c r="B69" s="9" t="inlineStr">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>26.8 KB</t>
+          <t>184.0 KB</t>
         </is>
       </c>
       <c r="E69" s="10" t="inlineStr">
@@ -2637,7 +2637,7 @@
     <row r="70" ht="16" customHeight="1">
       <c r="A70" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-09-_Y-32yPvO0k--16x9.jpg</t>
+          <t>images/comms-env-06-GP7SH7RRkqo--2x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B70" s="11" t="inlineStr">
@@ -2652,7 +2652,7 @@
       </c>
       <c r="D70" s="11" t="inlineStr">
         <is>
-          <t>39.7 KB</t>
+          <t>196.6 KB</t>
         </is>
       </c>
       <c r="E70" s="12" t="inlineStr">
@@ -2664,7 +2664,7 @@
     <row r="71" ht="16" customHeight="1">
       <c r="A71" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-09-_Y-32yPvO0k--1x1-textsafe.jpg</t>
+          <t>images/comms-env-06-GP7SH7RRkqo--2x1.jpg</t>
         </is>
       </c>
       <c r="B71" s="9" t="inlineStr">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>23.8 KB</t>
+          <t>260.4 KB</t>
         </is>
       </c>
       <c r="E71" s="10" t="inlineStr">
@@ -2691,7 +2691,7 @@
     <row r="72" ht="16" customHeight="1">
       <c r="A72" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-09-_Y-32yPvO0k--1x1.jpg</t>
+          <t>images/comms-env-06-GP7SH7RRkqo.jpg</t>
         </is>
       </c>
       <c r="B72" s="11" t="inlineStr">
@@ -2706,7 +2706,7 @@
       </c>
       <c r="D72" s="11" t="inlineStr">
         <is>
-          <t>35.3 KB</t>
+          <t>365.4 KB</t>
         </is>
       </c>
       <c r="E72" s="12" t="inlineStr">
@@ -2718,7 +2718,7 @@
     <row r="73" ht="16" customHeight="1">
       <c r="A73" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-09-_Y-32yPvO0k--2x1-textsafe.jpg</t>
+          <t>images/comms-env-07-qoJpt9Ja6y0--16x9-textsafe.jpg</t>
         </is>
       </c>
       <c r="B73" s="9" t="inlineStr">
@@ -2733,7 +2733,7 @@
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>24.2 KB</t>
+          <t>23.5 KB</t>
         </is>
       </c>
       <c r="E73" s="10" t="inlineStr">
@@ -2745,7 +2745,7 @@
     <row r="74" ht="16" customHeight="1">
       <c r="A74" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-09-_Y-32yPvO0k--2x1.jpg</t>
+          <t>images/comms-env-07-qoJpt9Ja6y0--16x9.jpg</t>
         </is>
       </c>
       <c r="B74" s="11" t="inlineStr">
@@ -2760,7 +2760,7 @@
       </c>
       <c r="D74" s="11" t="inlineStr">
         <is>
-          <t>36.3 KB</t>
+          <t>32.9 KB</t>
         </is>
       </c>
       <c r="E74" s="12" t="inlineStr">
@@ -2772,7 +2772,7 @@
     <row r="75" ht="16" customHeight="1">
       <c r="A75" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-09-_Y-32yPvO0k.jpg</t>
+          <t>images/comms-env-07-qoJpt9Ja6y0--1x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B75" s="9" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>54.9 KB</t>
+          <t>17.9 KB</t>
         </is>
       </c>
       <c r="E75" s="10" t="inlineStr">
@@ -2799,7 +2799,7 @@
     <row r="76" ht="16" customHeight="1">
       <c r="A76" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-10-N6jxoR1PcbE--16x9-textsafe.jpg</t>
+          <t>images/comms-env-07-qoJpt9Ja6y0--1x1.jpg</t>
         </is>
       </c>
       <c r="B76" s="11" t="inlineStr">
@@ -2814,7 +2814,7 @@
       </c>
       <c r="D76" s="11" t="inlineStr">
         <is>
-          <t>69.7 KB</t>
+          <t>25.5 KB</t>
         </is>
       </c>
       <c r="E76" s="12" t="inlineStr">
@@ -2826,7 +2826,7 @@
     <row r="77" ht="16" customHeight="1">
       <c r="A77" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-10-N6jxoR1PcbE--16x9.jpg</t>
+          <t>images/comms-env-07-qoJpt9Ja6y0--2x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B77" s="9" t="inlineStr">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>95.5 KB</t>
+          <t>22.0 KB</t>
         </is>
       </c>
       <c r="E77" s="10" t="inlineStr">
@@ -2853,7 +2853,7 @@
     <row r="78" ht="16" customHeight="1">
       <c r="A78" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-10-N6jxoR1PcbE--1x1-textsafe.jpg</t>
+          <t>images/comms-env-07-qoJpt9Ja6y0--2x1.jpg</t>
         </is>
       </c>
       <c r="B78" s="11" t="inlineStr">
@@ -2868,7 +2868,7 @@
       </c>
       <c r="D78" s="11" t="inlineStr">
         <is>
-          <t>58.1 KB</t>
+          <t>30.7 KB</t>
         </is>
       </c>
       <c r="E78" s="12" t="inlineStr">
@@ -2880,7 +2880,7 @@
     <row r="79" ht="16" customHeight="1">
       <c r="A79" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-10-N6jxoR1PcbE--1x1.jpg</t>
+          <t>images/comms-env-07-qoJpt9Ja6y0.jpg</t>
         </is>
       </c>
       <c r="B79" s="9" t="inlineStr">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>77.8 KB</t>
+          <t>40.9 KB</t>
         </is>
       </c>
       <c r="E79" s="10" t="inlineStr">
@@ -2907,7 +2907,7 @@
     <row r="80" ht="16" customHeight="1">
       <c r="A80" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-10-N6jxoR1PcbE--2x1-textsafe.jpg</t>
+          <t>images/comms-env-08-bGo01h57aCE--16x9-textsafe.jpg</t>
         </is>
       </c>
       <c r="B80" s="11" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="D80" s="11" t="inlineStr">
         <is>
-          <t>67.8 KB</t>
+          <t>84.0 KB</t>
         </is>
       </c>
       <c r="E80" s="12" t="inlineStr">
@@ -2934,7 +2934,7 @@
     <row r="81" ht="16" customHeight="1">
       <c r="A81" s="9" t="inlineStr">
         <is>
-          <t>images/comms-env-10-N6jxoR1PcbE--2x1.jpg</t>
+          <t>images/comms-env-08-bGo01h57aCE--16x9.jpg</t>
         </is>
       </c>
       <c r="B81" s="9" t="inlineStr">
@@ -2949,7 +2949,7 @@
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>92.2 KB</t>
+          <t>105.3 KB</t>
         </is>
       </c>
       <c r="E81" s="10" t="inlineStr">
@@ -2961,7 +2961,7 @@
     <row r="82" ht="16" customHeight="1">
       <c r="A82" s="11" t="inlineStr">
         <is>
-          <t>images/comms-env-10-N6jxoR1PcbE.jpg</t>
+          <t>images/comms-env-08-bGo01h57aCE--1x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B82" s="11" t="inlineStr">
@@ -2976,7 +2976,7 @@
       </c>
       <c r="D82" s="11" t="inlineStr">
         <is>
-          <t>120.1 KB</t>
+          <t>61.0 KB</t>
         </is>
       </c>
       <c r="E82" s="12" t="inlineStr">
@@ -2988,7 +2988,7 @@
     <row r="83" ht="16" customHeight="1">
       <c r="A83" s="9" t="inlineStr">
         <is>
-          <t>images/data-tex-01-OM1sIbjviw0--16x9-textsafe.jpg</t>
+          <t>images/comms-env-08-bGo01h57aCE--1x1.jpg</t>
         </is>
       </c>
       <c r="B83" s="9" t="inlineStr">
@@ -3003,7 +3003,7 @@
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>112.8 KB</t>
+          <t>75.6 KB</t>
         </is>
       </c>
       <c r="E83" s="10" t="inlineStr">
@@ -3015,7 +3015,7 @@
     <row r="84" ht="16" customHeight="1">
       <c r="A84" s="11" t="inlineStr">
         <is>
-          <t>images/data-tex-01-OM1sIbjviw0--16x9.jpg</t>
+          <t>images/comms-env-08-bGo01h57aCE--2x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B84" s="11" t="inlineStr">
@@ -3030,7 +3030,7 @@
       </c>
       <c r="D84" s="11" t="inlineStr">
         <is>
-          <t>167.7 KB</t>
+          <t>82.0 KB</t>
         </is>
       </c>
       <c r="E84" s="12" t="inlineStr">
@@ -3042,7 +3042,7 @@
     <row r="85" ht="16" customHeight="1">
       <c r="A85" s="9" t="inlineStr">
         <is>
-          <t>images/data-tex-01-OM1sIbjviw0--1x1-textsafe.jpg</t>
+          <t>images/comms-env-08-bGo01h57aCE--2x1.jpg</t>
         </is>
       </c>
       <c r="B85" s="9" t="inlineStr">
@@ -3057,7 +3057,7 @@
       </c>
       <c r="D85" s="9" t="inlineStr">
         <is>
-          <t>82.8 KB</t>
+          <t>101.9 KB</t>
         </is>
       </c>
       <c r="E85" s="10" t="inlineStr">
@@ -3069,7 +3069,7 @@
     <row r="86" ht="16" customHeight="1">
       <c r="A86" s="11" t="inlineStr">
         <is>
-          <t>images/data-tex-01-OM1sIbjviw0--1x1.jpg</t>
+          <t>images/comms-env-08-bGo01h57aCE.jpg</t>
         </is>
       </c>
       <c r="B86" s="11" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="D86" s="11" t="inlineStr">
         <is>
-          <t>122.5 KB</t>
+          <t>118.8 KB</t>
         </is>
       </c>
       <c r="E86" s="12" t="inlineStr">
@@ -3096,7 +3096,7 @@
     <row r="87" ht="16" customHeight="1">
       <c r="A87" s="9" t="inlineStr">
         <is>
-          <t>images/data-tex-01-OM1sIbjviw0--2x1-textsafe.jpg</t>
+          <t>images/comms-env-09-_Y-32yPvO0k--16x9-textsafe.jpg</t>
         </is>
       </c>
       <c r="B87" s="9" t="inlineStr">
@@ -3111,7 +3111,7 @@
       </c>
       <c r="D87" s="9" t="inlineStr">
         <is>
-          <t>100.0 KB</t>
+          <t>26.8 KB</t>
         </is>
       </c>
       <c r="E87" s="10" t="inlineStr">
@@ -3123,7 +3123,7 @@
     <row r="88" ht="16" customHeight="1">
       <c r="A88" s="11" t="inlineStr">
         <is>
-          <t>images/data-tex-01-OM1sIbjviw0--2x1.jpg</t>
+          <t>images/comms-env-09-_Y-32yPvO0k--16x9.jpg</t>
         </is>
       </c>
       <c r="B88" s="11" t="inlineStr">
@@ -3138,7 +3138,7 @@
       </c>
       <c r="D88" s="11" t="inlineStr">
         <is>
-          <t>149.2 KB</t>
+          <t>39.7 KB</t>
         </is>
       </c>
       <c r="E88" s="12" t="inlineStr">
@@ -3150,7 +3150,7 @@
     <row r="89" ht="16" customHeight="1">
       <c r="A89" s="9" t="inlineStr">
         <is>
-          <t>images/data-tex-01-OM1sIbjviw0.jpg</t>
+          <t>images/comms-env-09-_Y-32yPvO0k--1x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B89" s="9" t="inlineStr">
@@ -3165,7 +3165,7 @@
       </c>
       <c r="D89" s="9" t="inlineStr">
         <is>
-          <t>267.9 KB</t>
+          <t>23.8 KB</t>
         </is>
       </c>
       <c r="E89" s="10" t="inlineStr">
@@ -3177,7 +3177,7 @@
     <row r="90" ht="16" customHeight="1">
       <c r="A90" s="11" t="inlineStr">
         <is>
-          <t>images/data-tex-03-lTOM38wVEGM--16x9-textsafe.jpg</t>
+          <t>images/comms-env-09-_Y-32yPvO0k--1x1.jpg</t>
         </is>
       </c>
       <c r="B90" s="11" t="inlineStr">
@@ -3192,7 +3192,7 @@
       </c>
       <c r="D90" s="11" t="inlineStr">
         <is>
-          <t>111.0 KB</t>
+          <t>35.3 KB</t>
         </is>
       </c>
       <c r="E90" s="12" t="inlineStr">
@@ -3204,7 +3204,7 @@
     <row r="91" ht="16" customHeight="1">
       <c r="A91" s="9" t="inlineStr">
         <is>
-          <t>images/data-tex-03-lTOM38wVEGM--16x9.jpg</t>
+          <t>images/comms-env-09-_Y-32yPvO0k--2x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B91" s="9" t="inlineStr">
@@ -3219,7 +3219,7 @@
       </c>
       <c r="D91" s="9" t="inlineStr">
         <is>
-          <t>153.2 KB</t>
+          <t>24.2 KB</t>
         </is>
       </c>
       <c r="E91" s="10" t="inlineStr">
@@ -3231,7 +3231,7 @@
     <row r="92" ht="16" customHeight="1">
       <c r="A92" s="11" t="inlineStr">
         <is>
-          <t>images/data-tex-03-lTOM38wVEGM--1x1-textsafe.jpg</t>
+          <t>images/comms-env-09-_Y-32yPvO0k--2x1.jpg</t>
         </is>
       </c>
       <c r="B92" s="11" t="inlineStr">
@@ -3246,7 +3246,7 @@
       </c>
       <c r="D92" s="11" t="inlineStr">
         <is>
-          <t>78.3 KB</t>
+          <t>36.3 KB</t>
         </is>
       </c>
       <c r="E92" s="12" t="inlineStr">
@@ -3258,7 +3258,7 @@
     <row r="93" ht="16" customHeight="1">
       <c r="A93" s="9" t="inlineStr">
         <is>
-          <t>images/data-tex-03-lTOM38wVEGM--1x1.jpg</t>
+          <t>images/comms-env-09-_Y-32yPvO0k.jpg</t>
         </is>
       </c>
       <c r="B93" s="9" t="inlineStr">
@@ -3273,7 +3273,7 @@
       </c>
       <c r="D93" s="9" t="inlineStr">
         <is>
-          <t>108.2 KB</t>
+          <t>54.9 KB</t>
         </is>
       </c>
       <c r="E93" s="10" t="inlineStr">
@@ -3285,7 +3285,7 @@
     <row r="94" ht="16" customHeight="1">
       <c r="A94" s="11" t="inlineStr">
         <is>
-          <t>images/data-tex-03-lTOM38wVEGM--2x1-textsafe.jpg</t>
+          <t>images/comms-env-10-N6jxoR1PcbE--16x9-textsafe.jpg</t>
         </is>
       </c>
       <c r="B94" s="11" t="inlineStr">
@@ -3300,7 +3300,7 @@
       </c>
       <c r="D94" s="11" t="inlineStr">
         <is>
-          <t>100.5 KB</t>
+          <t>69.7 KB</t>
         </is>
       </c>
       <c r="E94" s="12" t="inlineStr">
@@ -3312,7 +3312,7 @@
     <row r="95" ht="16" customHeight="1">
       <c r="A95" s="9" t="inlineStr">
         <is>
-          <t>images/data-tex-03-lTOM38wVEGM--2x1.jpg</t>
+          <t>images/comms-env-10-N6jxoR1PcbE--16x9.jpg</t>
         </is>
       </c>
       <c r="B95" s="9" t="inlineStr">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="D95" s="9" t="inlineStr">
         <is>
-          <t>138.8 KB</t>
+          <t>95.5 KB</t>
         </is>
       </c>
       <c r="E95" s="10" t="inlineStr">
@@ -3339,7 +3339,7 @@
     <row r="96" ht="16" customHeight="1">
       <c r="A96" s="11" t="inlineStr">
         <is>
-          <t>images/data-tex-03-lTOM38wVEGM.jpg</t>
+          <t>images/comms-env-10-N6jxoR1PcbE--1x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B96" s="11" t="inlineStr">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="D96" s="11" t="inlineStr">
         <is>
-          <t>194.3 KB</t>
+          <t>58.1 KB</t>
         </is>
       </c>
       <c r="E96" s="12" t="inlineStr">
@@ -3366,7 +3366,7 @@
     <row r="97" ht="16" customHeight="1">
       <c r="A97" s="9" t="inlineStr">
         <is>
-          <t>images/data-tex-04-inHGrOADoVc--16x9-textsafe.jpg</t>
+          <t>images/comms-env-10-N6jxoR1PcbE--1x1.jpg</t>
         </is>
       </c>
       <c r="B97" s="9" t="inlineStr">
@@ -3381,7 +3381,7 @@
       </c>
       <c r="D97" s="9" t="inlineStr">
         <is>
-          <t>73.3 KB</t>
+          <t>77.8 KB</t>
         </is>
       </c>
       <c r="E97" s="10" t="inlineStr">
@@ -3393,7 +3393,7 @@
     <row r="98" ht="16" customHeight="1">
       <c r="A98" s="11" t="inlineStr">
         <is>
-          <t>images/data-tex-04-inHGrOADoVc--16x9.jpg</t>
+          <t>images/comms-env-10-N6jxoR1PcbE--2x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B98" s="11" t="inlineStr">
@@ -3408,7 +3408,7 @@
       </c>
       <c r="D98" s="11" t="inlineStr">
         <is>
-          <t>103.9 KB</t>
+          <t>67.8 KB</t>
         </is>
       </c>
       <c r="E98" s="12" t="inlineStr">
@@ -3420,7 +3420,7 @@
     <row r="99" ht="16" customHeight="1">
       <c r="A99" s="9" t="inlineStr">
         <is>
-          <t>images/data-tex-04-inHGrOADoVc--1x1-textsafe.jpg</t>
+          <t>images/comms-env-10-N6jxoR1PcbE--2x1.jpg</t>
         </is>
       </c>
       <c r="B99" s="9" t="inlineStr">
@@ -3435,7 +3435,7 @@
       </c>
       <c r="D99" s="9" t="inlineStr">
         <is>
-          <t>54.2 KB</t>
+          <t>92.2 KB</t>
         </is>
       </c>
       <c r="E99" s="10" t="inlineStr">
@@ -3447,7 +3447,7 @@
     <row r="100" ht="16" customHeight="1">
       <c r="A100" s="11" t="inlineStr">
         <is>
-          <t>images/data-tex-04-inHGrOADoVc--1x1.jpg</t>
+          <t>images/comms-env-10-N6jxoR1PcbE.jpg</t>
         </is>
       </c>
       <c r="B100" s="11" t="inlineStr">
@@ -3462,7 +3462,7 @@
       </c>
       <c r="D100" s="11" t="inlineStr">
         <is>
-          <t>75.8 KB</t>
+          <t>120.1 KB</t>
         </is>
       </c>
       <c r="E100" s="12" t="inlineStr">
@@ -3474,7 +3474,7 @@
     <row r="101" ht="16" customHeight="1">
       <c r="A101" s="9" t="inlineStr">
         <is>
-          <t>images/data-tex-04-inHGrOADoVc--2x1-textsafe.jpg</t>
+          <t>images/data-tex-01-OM1sIbjviw0--16x9-textsafe.jpg</t>
         </is>
       </c>
       <c r="B101" s="9" t="inlineStr">
@@ -3489,7 +3489,7 @@
       </c>
       <c r="D101" s="9" t="inlineStr">
         <is>
-          <t>63.7 KB</t>
+          <t>112.8 KB</t>
         </is>
       </c>
       <c r="E101" s="10" t="inlineStr">
@@ -3501,7 +3501,7 @@
     <row r="102" ht="16" customHeight="1">
       <c r="A102" s="11" t="inlineStr">
         <is>
-          <t>images/data-tex-04-inHGrOADoVc--2x1.jpg</t>
+          <t>images/data-tex-01-OM1sIbjviw0--16x9.jpg</t>
         </is>
       </c>
       <c r="B102" s="11" t="inlineStr">
@@ -3516,7 +3516,7 @@
       </c>
       <c r="D102" s="11" t="inlineStr">
         <is>
-          <t>91.0 KB</t>
+          <t>167.7 KB</t>
         </is>
       </c>
       <c r="E102" s="12" t="inlineStr">
@@ -3528,7 +3528,7 @@
     <row r="103" ht="16" customHeight="1">
       <c r="A103" s="9" t="inlineStr">
         <is>
-          <t>images/data-tex-04-inHGrOADoVc.jpg</t>
+          <t>images/data-tex-01-OM1sIbjviw0--1x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B103" s="9" t="inlineStr">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="D103" s="9" t="inlineStr">
         <is>
-          <t>151.9 KB</t>
+          <t>82.8 KB</t>
         </is>
       </c>
       <c r="E103" s="10" t="inlineStr">
@@ -3555,7 +3555,7 @@
     <row r="104" ht="16" customHeight="1">
       <c r="A104" s="11" t="inlineStr">
         <is>
-          <t>images/data-tex-05-ETiSF2VSRTQ--16x9-textsafe.jpg</t>
+          <t>images/data-tex-01-OM1sIbjviw0--1x1.jpg</t>
         </is>
       </c>
       <c r="B104" s="11" t="inlineStr">
@@ -3570,7 +3570,7 @@
       </c>
       <c r="D104" s="11" t="inlineStr">
         <is>
-          <t>50.2 KB</t>
+          <t>122.5 KB</t>
         </is>
       </c>
       <c r="E104" s="12" t="inlineStr">
@@ -3582,7 +3582,7 @@
     <row r="105" ht="16" customHeight="1">
       <c r="A105" s="9" t="inlineStr">
         <is>
-          <t>images/data-tex-05-ETiSF2VSRTQ--16x9.jpg</t>
+          <t>images/data-tex-01-OM1sIbjviw0--2x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B105" s="9" t="inlineStr">
@@ -3597,7 +3597,7 @@
       </c>
       <c r="D105" s="9" t="inlineStr">
         <is>
-          <t>83.5 KB</t>
+          <t>100.0 KB</t>
         </is>
       </c>
       <c r="E105" s="10" t="inlineStr">
@@ -3609,7 +3609,7 @@
     <row r="106" ht="16" customHeight="1">
       <c r="A106" s="11" t="inlineStr">
         <is>
-          <t>images/data-tex-05-ETiSF2VSRTQ--1x1-textsafe.jpg</t>
+          <t>images/data-tex-01-OM1sIbjviw0--2x1.jpg</t>
         </is>
       </c>
       <c r="B106" s="11" t="inlineStr">
@@ -3624,7 +3624,7 @@
       </c>
       <c r="D106" s="11" t="inlineStr">
         <is>
-          <t>39.1 KB</t>
+          <t>149.2 KB</t>
         </is>
       </c>
       <c r="E106" s="12" t="inlineStr">
@@ -3636,7 +3636,7 @@
     <row r="107" ht="16" customHeight="1">
       <c r="A107" s="9" t="inlineStr">
         <is>
-          <t>images/data-tex-05-ETiSF2VSRTQ--1x1.jpg</t>
+          <t>images/data-tex-01-OM1sIbjviw0.jpg</t>
         </is>
       </c>
       <c r="B107" s="9" t="inlineStr">
@@ -3651,7 +3651,7 @@
       </c>
       <c r="D107" s="9" t="inlineStr">
         <is>
-          <t>64.6 KB</t>
+          <t>267.9 KB</t>
         </is>
       </c>
       <c r="E107" s="10" t="inlineStr">
@@ -3663,7 +3663,7 @@
     <row r="108" ht="16" customHeight="1">
       <c r="A108" s="11" t="inlineStr">
         <is>
-          <t>images/data-tex-05-ETiSF2VSRTQ--2x1-textsafe.jpg</t>
+          <t>images/data-tex-03-lTOM38wVEGM--16x9-textsafe.jpg</t>
         </is>
       </c>
       <c r="B108" s="11" t="inlineStr">
@@ -3678,7 +3678,7 @@
       </c>
       <c r="D108" s="11" t="inlineStr">
         <is>
-          <t>44.8 KB</t>
+          <t>111.0 KB</t>
         </is>
       </c>
       <c r="E108" s="12" t="inlineStr">
@@ -3690,7 +3690,7 @@
     <row r="109" ht="16" customHeight="1">
       <c r="A109" s="9" t="inlineStr">
         <is>
-          <t>images/data-tex-05-ETiSF2VSRTQ--2x1.jpg</t>
+          <t>images/data-tex-03-lTOM38wVEGM--16x9.jpg</t>
         </is>
       </c>
       <c r="B109" s="9" t="inlineStr">
@@ -3705,7 +3705,7 @@
       </c>
       <c r="D109" s="9" t="inlineStr">
         <is>
-          <t>74.3 KB</t>
+          <t>153.2 KB</t>
         </is>
       </c>
       <c r="E109" s="10" t="inlineStr">
@@ -3717,7 +3717,7 @@
     <row r="110" ht="16" customHeight="1">
       <c r="A110" s="11" t="inlineStr">
         <is>
-          <t>images/data-tex-05-ETiSF2VSRTQ.jpg</t>
+          <t>images/data-tex-03-lTOM38wVEGM--1x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B110" s="11" t="inlineStr">
@@ -3732,7 +3732,7 @@
       </c>
       <c r="D110" s="11" t="inlineStr">
         <is>
-          <t>114.2 KB</t>
+          <t>78.3 KB</t>
         </is>
       </c>
       <c r="E110" s="12" t="inlineStr">
@@ -3744,7 +3744,7 @@
     <row r="111" ht="16" customHeight="1">
       <c r="A111" s="9" t="inlineStr">
         <is>
-          <t>images/judgment-01-0_OlKblZ4eY--16x9-textsafe.jpg</t>
+          <t>images/data-tex-03-lTOM38wVEGM--1x1.jpg</t>
         </is>
       </c>
       <c r="B111" s="9" t="inlineStr">
@@ -3759,7 +3759,7 @@
       </c>
       <c r="D111" s="9" t="inlineStr">
         <is>
-          <t>61.4 KB</t>
+          <t>108.2 KB</t>
         </is>
       </c>
       <c r="E111" s="10" t="inlineStr">
@@ -3771,7 +3771,7 @@
     <row r="112" ht="16" customHeight="1">
       <c r="A112" s="11" t="inlineStr">
         <is>
-          <t>images/judgment-01-0_OlKblZ4eY--16x9.jpg</t>
+          <t>images/data-tex-03-lTOM38wVEGM--2x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B112" s="11" t="inlineStr">
@@ -3786,7 +3786,7 @@
       </c>
       <c r="D112" s="11" t="inlineStr">
         <is>
-          <t>99.4 KB</t>
+          <t>100.5 KB</t>
         </is>
       </c>
       <c r="E112" s="12" t="inlineStr">
@@ -3798,7 +3798,7 @@
     <row r="113" ht="16" customHeight="1">
       <c r="A113" s="9" t="inlineStr">
         <is>
-          <t>images/judgment-01-0_OlKblZ4eY--1x1-textsafe.jpg</t>
+          <t>images/data-tex-03-lTOM38wVEGM--2x1.jpg</t>
         </is>
       </c>
       <c r="B113" s="9" t="inlineStr">
@@ -3813,7 +3813,7 @@
       </c>
       <c r="D113" s="9" t="inlineStr">
         <is>
-          <t>48.7 KB</t>
+          <t>138.8 KB</t>
         </is>
       </c>
       <c r="E113" s="10" t="inlineStr">
@@ -3825,7 +3825,7 @@
     <row r="114" ht="16" customHeight="1">
       <c r="A114" s="11" t="inlineStr">
         <is>
-          <t>images/judgment-01-0_OlKblZ4eY--1x1.jpg</t>
+          <t>images/data-tex-03-lTOM38wVEGM.jpg</t>
         </is>
       </c>
       <c r="B114" s="11" t="inlineStr">
@@ -3840,7 +3840,7 @@
       </c>
       <c r="D114" s="11" t="inlineStr">
         <is>
-          <t>77.3 KB</t>
+          <t>194.3 KB</t>
         </is>
       </c>
       <c r="E114" s="12" t="inlineStr">
@@ -3852,7 +3852,7 @@
     <row r="115" ht="16" customHeight="1">
       <c r="A115" s="9" t="inlineStr">
         <is>
-          <t>images/judgment-01-0_OlKblZ4eY--2x1-textsafe.jpg</t>
+          <t>images/data-tex-04-inHGrOADoVc--16x9-textsafe.jpg</t>
         </is>
       </c>
       <c r="B115" s="9" t="inlineStr">
@@ -3867,7 +3867,7 @@
       </c>
       <c r="D115" s="9" t="inlineStr">
         <is>
-          <t>55.7 KB</t>
+          <t>73.3 KB</t>
         </is>
       </c>
       <c r="E115" s="10" t="inlineStr">
@@ -3879,7 +3879,7 @@
     <row r="116" ht="16" customHeight="1">
       <c r="A116" s="11" t="inlineStr">
         <is>
-          <t>images/judgment-01-0_OlKblZ4eY--2x1.jpg</t>
+          <t>images/data-tex-04-inHGrOADoVc--16x9.jpg</t>
         </is>
       </c>
       <c r="B116" s="11" t="inlineStr">
@@ -3894,7 +3894,7 @@
       </c>
       <c r="D116" s="11" t="inlineStr">
         <is>
-          <t>90.1 KB</t>
+          <t>103.9 KB</t>
         </is>
       </c>
       <c r="E116" s="12" t="inlineStr">
@@ -3906,7 +3906,7 @@
     <row r="117" ht="16" customHeight="1">
       <c r="A117" s="9" t="inlineStr">
         <is>
-          <t>images/judgment-01-0_OlKblZ4eY.jpg</t>
+          <t>images/data-tex-04-inHGrOADoVc--1x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B117" s="9" t="inlineStr">
@@ -3921,7 +3921,7 @@
       </c>
       <c r="D117" s="9" t="inlineStr">
         <is>
-          <t>156.3 KB</t>
+          <t>54.2 KB</t>
         </is>
       </c>
       <c r="E117" s="10" t="inlineStr">
@@ -3933,7 +3933,7 @@
     <row r="118" ht="16" customHeight="1">
       <c r="A118" s="11" t="inlineStr">
         <is>
-          <t>images/judgment-03-ii-Vf8dahfo--16x9-textsafe.jpg</t>
+          <t>images/data-tex-04-inHGrOADoVc--1x1.jpg</t>
         </is>
       </c>
       <c r="B118" s="11" t="inlineStr">
@@ -3948,7 +3948,7 @@
       </c>
       <c r="D118" s="11" t="inlineStr">
         <is>
-          <t>70.5 KB</t>
+          <t>75.8 KB</t>
         </is>
       </c>
       <c r="E118" s="12" t="inlineStr">
@@ -3960,7 +3960,7 @@
     <row r="119" ht="16" customHeight="1">
       <c r="A119" s="9" t="inlineStr">
         <is>
-          <t>images/judgment-03-ii-Vf8dahfo--16x9.jpg</t>
+          <t>images/data-tex-04-inHGrOADoVc--2x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B119" s="9" t="inlineStr">
@@ -3975,7 +3975,7 @@
       </c>
       <c r="D119" s="9" t="inlineStr">
         <is>
-          <t>123.9 KB</t>
+          <t>63.7 KB</t>
         </is>
       </c>
       <c r="E119" s="10" t="inlineStr">
@@ -3987,7 +3987,7 @@
     <row r="120" ht="16" customHeight="1">
       <c r="A120" s="11" t="inlineStr">
         <is>
-          <t>images/judgment-03-ii-Vf8dahfo--1x1-textsafe.jpg</t>
+          <t>images/data-tex-04-inHGrOADoVc--2x1.jpg</t>
         </is>
       </c>
       <c r="B120" s="11" t="inlineStr">
@@ -4002,7 +4002,7 @@
       </c>
       <c r="D120" s="11" t="inlineStr">
         <is>
-          <t>57.5 KB</t>
+          <t>91.0 KB</t>
         </is>
       </c>
       <c r="E120" s="12" t="inlineStr">
@@ -4014,7 +4014,7 @@
     <row r="121" ht="16" customHeight="1">
       <c r="A121" s="9" t="inlineStr">
         <is>
-          <t>images/judgment-03-ii-Vf8dahfo--1x1.jpg</t>
+          <t>images/data-tex-04-inHGrOADoVc.jpg</t>
         </is>
       </c>
       <c r="B121" s="9" t="inlineStr">
@@ -4029,7 +4029,7 @@
       </c>
       <c r="D121" s="9" t="inlineStr">
         <is>
-          <t>93.8 KB</t>
+          <t>151.9 KB</t>
         </is>
       </c>
       <c r="E121" s="10" t="inlineStr">
@@ -4041,7 +4041,7 @@
     <row r="122" ht="16" customHeight="1">
       <c r="A122" s="11" t="inlineStr">
         <is>
-          <t>images/judgment-03-ii-Vf8dahfo--2x1-textsafe.jpg</t>
+          <t>images/data-tex-05-ETiSF2VSRTQ--16x9-textsafe.jpg</t>
         </is>
       </c>
       <c r="B122" s="11" t="inlineStr">
@@ -4056,7 +4056,7 @@
       </c>
       <c r="D122" s="11" t="inlineStr">
         <is>
-          <t>63.4 KB</t>
+          <t>50.2 KB</t>
         </is>
       </c>
       <c r="E122" s="12" t="inlineStr">
@@ -4068,7 +4068,7 @@
     <row r="123" ht="16" customHeight="1">
       <c r="A123" s="9" t="inlineStr">
         <is>
-          <t>images/judgment-03-ii-Vf8dahfo--2x1.jpg</t>
+          <t>images/data-tex-05-ETiSF2VSRTQ--16x9.jpg</t>
         </is>
       </c>
       <c r="B123" s="9" t="inlineStr">
@@ -4083,7 +4083,7 @@
       </c>
       <c r="D123" s="9" t="inlineStr">
         <is>
-          <t>111.8 KB</t>
+          <t>83.5 KB</t>
         </is>
       </c>
       <c r="E123" s="10" t="inlineStr">
@@ -4095,7 +4095,7 @@
     <row r="124" ht="16" customHeight="1">
       <c r="A124" s="11" t="inlineStr">
         <is>
-          <t>images/judgment-03-ii-Vf8dahfo.jpg</t>
+          <t>images/data-tex-05-ETiSF2VSRTQ--1x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B124" s="11" t="inlineStr">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="D124" s="11" t="inlineStr">
         <is>
-          <t>168.1 KB</t>
+          <t>39.1 KB</t>
         </is>
       </c>
       <c r="E124" s="12" t="inlineStr">
@@ -4122,7 +4122,7 @@
     <row r="125" ht="16" customHeight="1">
       <c r="A125" s="9" t="inlineStr">
         <is>
-          <t>images/judgment-04-ocfQmiQAuBo--16x9-textsafe.jpg</t>
+          <t>images/data-tex-05-ETiSF2VSRTQ--1x1.jpg</t>
         </is>
       </c>
       <c r="B125" s="9" t="inlineStr">
@@ -4137,7 +4137,7 @@
       </c>
       <c r="D125" s="9" t="inlineStr">
         <is>
-          <t>72.5 KB</t>
+          <t>64.6 KB</t>
         </is>
       </c>
       <c r="E125" s="10" t="inlineStr">
@@ -4149,7 +4149,7 @@
     <row r="126" ht="16" customHeight="1">
       <c r="A126" s="11" t="inlineStr">
         <is>
-          <t>images/judgment-04-ocfQmiQAuBo--16x9.jpg</t>
+          <t>images/data-tex-05-ETiSF2VSRTQ--2x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B126" s="11" t="inlineStr">
@@ -4164,7 +4164,7 @@
       </c>
       <c r="D126" s="11" t="inlineStr">
         <is>
-          <t>117.9 KB</t>
+          <t>44.8 KB</t>
         </is>
       </c>
       <c r="E126" s="12" t="inlineStr">
@@ -4176,7 +4176,7 @@
     <row r="127" ht="16" customHeight="1">
       <c r="A127" s="9" t="inlineStr">
         <is>
-          <t>images/judgment-04-ocfQmiQAuBo--1x1-textsafe.jpg</t>
+          <t>images/data-tex-05-ETiSF2VSRTQ--2x1.jpg</t>
         </is>
       </c>
       <c r="B127" s="9" t="inlineStr">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="D127" s="9" t="inlineStr">
         <is>
-          <t>53.9 KB</t>
+          <t>74.3 KB</t>
         </is>
       </c>
       <c r="E127" s="10" t="inlineStr">
@@ -4203,7 +4203,7 @@
     <row r="128" ht="16" customHeight="1">
       <c r="A128" s="11" t="inlineStr">
         <is>
-          <t>images/judgment-04-ocfQmiQAuBo--1x1.jpg</t>
+          <t>images/data-tex-05-ETiSF2VSRTQ.jpg</t>
         </is>
       </c>
       <c r="B128" s="11" t="inlineStr">
@@ -4218,7 +4218,7 @@
       </c>
       <c r="D128" s="11" t="inlineStr">
         <is>
-          <t>84.7 KB</t>
+          <t>114.2 KB</t>
         </is>
       </c>
       <c r="E128" s="12" t="inlineStr">
@@ -4230,7 +4230,7 @@
     <row r="129" ht="16" customHeight="1">
       <c r="A129" s="9" t="inlineStr">
         <is>
-          <t>images/judgment-04-ocfQmiQAuBo--2x1-textsafe.jpg</t>
+          <t>images/judgment-01-0_OlKblZ4eY--16x9-textsafe.jpg</t>
         </is>
       </c>
       <c r="B129" s="9" t="inlineStr">
@@ -4245,7 +4245,7 @@
       </c>
       <c r="D129" s="9" t="inlineStr">
         <is>
-          <t>67.3 KB</t>
+          <t>61.4 KB</t>
         </is>
       </c>
       <c r="E129" s="10" t="inlineStr">
@@ -4257,7 +4257,7 @@
     <row r="130" ht="16" customHeight="1">
       <c r="A130" s="11" t="inlineStr">
         <is>
-          <t>images/judgment-04-ocfQmiQAuBo--2x1.jpg</t>
+          <t>images/judgment-01-0_OlKblZ4eY--16x9.jpg</t>
         </is>
       </c>
       <c r="B130" s="11" t="inlineStr">
@@ -4272,7 +4272,7 @@
       </c>
       <c r="D130" s="11" t="inlineStr">
         <is>
-          <t>108.5 KB</t>
+          <t>99.4 KB</t>
         </is>
       </c>
       <c r="E130" s="12" t="inlineStr">
@@ -4284,7 +4284,7 @@
     <row r="131" ht="16" customHeight="1">
       <c r="A131" s="9" t="inlineStr">
         <is>
-          <t>images/judgment-04-ocfQmiQAuBo.jpg</t>
+          <t>images/judgment-01-0_OlKblZ4eY--1x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B131" s="9" t="inlineStr">
@@ -4299,7 +4299,7 @@
       </c>
       <c r="D131" s="9" t="inlineStr">
         <is>
-          <t>154.6 KB</t>
+          <t>48.7 KB</t>
         </is>
       </c>
       <c r="E131" s="10" t="inlineStr">
@@ -4311,7 +4311,7 @@
     <row r="132" ht="16" customHeight="1">
       <c r="A132" s="11" t="inlineStr">
         <is>
-          <t>images/judgment-05-Y1Dd_ASy9tc--16x9-textsafe.jpg</t>
+          <t>images/judgment-01-0_OlKblZ4eY--1x1.jpg</t>
         </is>
       </c>
       <c r="B132" s="11" t="inlineStr">
@@ -4326,7 +4326,7 @@
       </c>
       <c r="D132" s="11" t="inlineStr">
         <is>
-          <t>180.2 KB</t>
+          <t>77.3 KB</t>
         </is>
       </c>
       <c r="E132" s="12" t="inlineStr">
@@ -4338,7 +4338,7 @@
     <row r="133" ht="16" customHeight="1">
       <c r="A133" s="9" t="inlineStr">
         <is>
-          <t>images/judgment-05-Y1Dd_ASy9tc--16x9.jpg</t>
+          <t>images/judgment-01-0_OlKblZ4eY--2x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B133" s="9" t="inlineStr">
@@ -4353,7 +4353,7 @@
       </c>
       <c r="D133" s="9" t="inlineStr">
         <is>
-          <t>236.0 KB</t>
+          <t>55.7 KB</t>
         </is>
       </c>
       <c r="E133" s="10" t="inlineStr">
@@ -4365,7 +4365,7 @@
     <row r="134" ht="16" customHeight="1">
       <c r="A134" s="11" t="inlineStr">
         <is>
-          <t>images/judgment-05-Y1Dd_ASy9tc--1x1-textsafe.jpg</t>
+          <t>images/judgment-01-0_OlKblZ4eY--2x1.jpg</t>
         </is>
       </c>
       <c r="B134" s="11" t="inlineStr">
@@ -4380,7 +4380,7 @@
       </c>
       <c r="D134" s="11" t="inlineStr">
         <is>
-          <t>122.0 KB</t>
+          <t>90.1 KB</t>
         </is>
       </c>
       <c r="E134" s="12" t="inlineStr">
@@ -4392,7 +4392,7 @@
     <row r="135" ht="16" customHeight="1">
       <c r="A135" s="9" t="inlineStr">
         <is>
-          <t>images/judgment-05-Y1Dd_ASy9tc--1x1.jpg</t>
+          <t>images/judgment-01-0_OlKblZ4eY.jpg</t>
         </is>
       </c>
       <c r="B135" s="9" t="inlineStr">
@@ -4407,7 +4407,7 @@
       </c>
       <c r="D135" s="9" t="inlineStr">
         <is>
-          <t>159.9 KB</t>
+          <t>156.3 KB</t>
         </is>
       </c>
       <c r="E135" s="10" t="inlineStr">
@@ -4419,7 +4419,7 @@
     <row r="136" ht="16" customHeight="1">
       <c r="A136" s="11" t="inlineStr">
         <is>
-          <t>images/judgment-05-Y1Dd_ASy9tc--2x1-textsafe.jpg</t>
+          <t>images/judgment-03-ii-Vf8dahfo--16x9-textsafe.jpg</t>
         </is>
       </c>
       <c r="B136" s="11" t="inlineStr">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="D136" s="11" t="inlineStr">
         <is>
-          <t>166.3 KB</t>
+          <t>70.5 KB</t>
         </is>
       </c>
       <c r="E136" s="12" t="inlineStr">
@@ -4446,7 +4446,7 @@
     <row r="137" ht="16" customHeight="1">
       <c r="A137" s="9" t="inlineStr">
         <is>
-          <t>images/judgment-05-Y1Dd_ASy9tc--2x1.jpg</t>
+          <t>images/judgment-03-ii-Vf8dahfo--16x9.jpg</t>
         </is>
       </c>
       <c r="B137" s="9" t="inlineStr">
@@ -4461,7 +4461,7 @@
       </c>
       <c r="D137" s="9" t="inlineStr">
         <is>
-          <t>217.0 KB</t>
+          <t>123.9 KB</t>
         </is>
       </c>
       <c r="E137" s="10" t="inlineStr">
@@ -4473,7 +4473,7 @@
     <row r="138" ht="16" customHeight="1">
       <c r="A138" s="11" t="inlineStr">
         <is>
-          <t>images/judgment-05-Y1Dd_ASy9tc.jpg</t>
+          <t>images/judgment-03-ii-Vf8dahfo--1x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B138" s="11" t="inlineStr">
@@ -4488,7 +4488,7 @@
       </c>
       <c r="D138" s="11" t="inlineStr">
         <is>
-          <t>300.7 KB</t>
+          <t>57.5 KB</t>
         </is>
       </c>
       <c r="E138" s="12" t="inlineStr">
@@ -4500,7 +4500,7 @@
     <row r="139" ht="16" customHeight="1">
       <c r="A139" s="9" t="inlineStr">
         <is>
-          <t>images/signal-01-ux0tBq3xB60--16x9-textsafe.jpg</t>
+          <t>images/judgment-03-ii-Vf8dahfo--1x1.jpg</t>
         </is>
       </c>
       <c r="B139" s="9" t="inlineStr">
@@ -4515,7 +4515,7 @@
       </c>
       <c r="D139" s="9" t="inlineStr">
         <is>
-          <t>46.1 KB</t>
+          <t>93.8 KB</t>
         </is>
       </c>
       <c r="E139" s="10" t="inlineStr">
@@ -4527,7 +4527,7 @@
     <row r="140" ht="16" customHeight="1">
       <c r="A140" s="11" t="inlineStr">
         <is>
-          <t>images/signal-01-ux0tBq3xB60--16x9.jpg</t>
+          <t>images/judgment-03-ii-Vf8dahfo--2x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B140" s="11" t="inlineStr">
@@ -4542,7 +4542,7 @@
       </c>
       <c r="D140" s="11" t="inlineStr">
         <is>
-          <t>64.6 KB</t>
+          <t>63.4 KB</t>
         </is>
       </c>
       <c r="E140" s="12" t="inlineStr">
@@ -4554,7 +4554,7 @@
     <row r="141" ht="16" customHeight="1">
       <c r="A141" s="9" t="inlineStr">
         <is>
-          <t>images/signal-01-ux0tBq3xB60--1x1-textsafe.jpg</t>
+          <t>images/judgment-03-ii-Vf8dahfo--2x1.jpg</t>
         </is>
       </c>
       <c r="B141" s="9" t="inlineStr">
@@ -4569,7 +4569,7 @@
       </c>
       <c r="D141" s="9" t="inlineStr">
         <is>
-          <t>38.3 KB</t>
+          <t>111.8 KB</t>
         </is>
       </c>
       <c r="E141" s="10" t="inlineStr">
@@ -4581,7 +4581,7 @@
     <row r="142" ht="16" customHeight="1">
       <c r="A142" s="11" t="inlineStr">
         <is>
-          <t>images/signal-01-ux0tBq3xB60--1x1.jpg</t>
+          <t>images/judgment-03-ii-Vf8dahfo.jpg</t>
         </is>
       </c>
       <c r="B142" s="11" t="inlineStr">
@@ -4596,7 +4596,7 @@
       </c>
       <c r="D142" s="11" t="inlineStr">
         <is>
-          <t>52.7 KB</t>
+          <t>168.1 KB</t>
         </is>
       </c>
       <c r="E142" s="12" t="inlineStr">
@@ -4608,7 +4608,7 @@
     <row r="143" ht="16" customHeight="1">
       <c r="A143" s="9" t="inlineStr">
         <is>
-          <t>images/signal-01-ux0tBq3xB60--2x1-textsafe.jpg</t>
+          <t>images/judgment-04-ocfQmiQAuBo--16x9-textsafe.jpg</t>
         </is>
       </c>
       <c r="B143" s="9" t="inlineStr">
@@ -4623,7 +4623,7 @@
       </c>
       <c r="D143" s="9" t="inlineStr">
         <is>
-          <t>40.9 KB</t>
+          <t>72.5 KB</t>
         </is>
       </c>
       <c r="E143" s="10" t="inlineStr">
@@ -4635,7 +4635,7 @@
     <row r="144" ht="16" customHeight="1">
       <c r="A144" s="11" t="inlineStr">
         <is>
-          <t>images/signal-01-ux0tBq3xB60--2x1.jpg</t>
+          <t>images/judgment-04-ocfQmiQAuBo--16x9.jpg</t>
         </is>
       </c>
       <c r="B144" s="11" t="inlineStr">
@@ -4650,7 +4650,7 @@
       </c>
       <c r="D144" s="11" t="inlineStr">
         <is>
-          <t>57.4 KB</t>
+          <t>117.9 KB</t>
         </is>
       </c>
       <c r="E144" s="12" t="inlineStr">
@@ -4662,7 +4662,7 @@
     <row r="145" ht="16" customHeight="1">
       <c r="A145" s="9" t="inlineStr">
         <is>
-          <t>images/signal-01-ux0tBq3xB60.jpg</t>
+          <t>images/judgment-04-ocfQmiQAuBo--1x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B145" s="9" t="inlineStr">
@@ -4677,7 +4677,7 @@
       </c>
       <c r="D145" s="9" t="inlineStr">
         <is>
-          <t>103.1 KB</t>
+          <t>53.9 KB</t>
         </is>
       </c>
       <c r="E145" s="10" t="inlineStr">
@@ -4689,7 +4689,7 @@
     <row r="146" ht="16" customHeight="1">
       <c r="A146" s="11" t="inlineStr">
         <is>
-          <t>images/signal-02-5RQyZZytm-Y--16x9-textsafe.jpg</t>
+          <t>images/judgment-04-ocfQmiQAuBo--1x1.jpg</t>
         </is>
       </c>
       <c r="B146" s="11" t="inlineStr">
@@ -4704,7 +4704,7 @@
       </c>
       <c r="D146" s="11" t="inlineStr">
         <is>
-          <t>32.8 KB</t>
+          <t>84.7 KB</t>
         </is>
       </c>
       <c r="E146" s="12" t="inlineStr">
@@ -4716,7 +4716,7 @@
     <row r="147" ht="16" customHeight="1">
       <c r="A147" s="9" t="inlineStr">
         <is>
-          <t>images/signal-02-5RQyZZytm-Y--16x9.jpg</t>
+          <t>images/judgment-04-ocfQmiQAuBo--2x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B147" s="9" t="inlineStr">
@@ -4731,7 +4731,7 @@
       </c>
       <c r="D147" s="9" t="inlineStr">
         <is>
-          <t>53.9 KB</t>
+          <t>67.3 KB</t>
         </is>
       </c>
       <c r="E147" s="10" t="inlineStr">
@@ -4743,7 +4743,7 @@
     <row r="148" ht="16" customHeight="1">
       <c r="A148" s="11" t="inlineStr">
         <is>
-          <t>images/signal-02-5RQyZZytm-Y--1x1-textsafe.jpg</t>
+          <t>images/judgment-04-ocfQmiQAuBo--2x1.jpg</t>
         </is>
       </c>
       <c r="B148" s="11" t="inlineStr">
@@ -4758,7 +4758,7 @@
       </c>
       <c r="D148" s="11" t="inlineStr">
         <is>
-          <t>24.6 KB</t>
+          <t>108.5 KB</t>
         </is>
       </c>
       <c r="E148" s="12" t="inlineStr">
@@ -4770,7 +4770,7 @@
     <row r="149" ht="16" customHeight="1">
       <c r="A149" s="9" t="inlineStr">
         <is>
-          <t>images/signal-02-5RQyZZytm-Y--1x1.jpg</t>
+          <t>images/judgment-04-ocfQmiQAuBo.jpg</t>
         </is>
       </c>
       <c r="B149" s="9" t="inlineStr">
@@ -4785,7 +4785,7 @@
       </c>
       <c r="D149" s="9" t="inlineStr">
         <is>
-          <t>39.5 KB</t>
+          <t>154.6 KB</t>
         </is>
       </c>
       <c r="E149" s="10" t="inlineStr">
@@ -4797,7 +4797,7 @@
     <row r="150" ht="16" customHeight="1">
       <c r="A150" s="11" t="inlineStr">
         <is>
-          <t>images/signal-02-5RQyZZytm-Y--2x1-textsafe.jpg</t>
+          <t>images/judgment-05-Y1Dd_ASy9tc--16x9-textsafe.jpg</t>
         </is>
       </c>
       <c r="B150" s="11" t="inlineStr">
@@ -4812,7 +4812,7 @@
       </c>
       <c r="D150" s="11" t="inlineStr">
         <is>
-          <t>29.6 KB</t>
+          <t>180.2 KB</t>
         </is>
       </c>
       <c r="E150" s="12" t="inlineStr">
@@ -4824,7 +4824,7 @@
     <row r="151" ht="16" customHeight="1">
       <c r="A151" s="9" t="inlineStr">
         <is>
-          <t>images/signal-02-5RQyZZytm-Y--2x1.jpg</t>
+          <t>images/judgment-05-Y1Dd_ASy9tc--16x9.jpg</t>
         </is>
       </c>
       <c r="B151" s="9" t="inlineStr">
@@ -4839,7 +4839,7 @@
       </c>
       <c r="D151" s="9" t="inlineStr">
         <is>
-          <t>48.3 KB</t>
+          <t>236.0 KB</t>
         </is>
       </c>
       <c r="E151" s="10" t="inlineStr">
@@ -4851,7 +4851,7 @@
     <row r="152" ht="16" customHeight="1">
       <c r="A152" s="11" t="inlineStr">
         <is>
-          <t>images/signal-02-5RQyZZytm-Y.jpg</t>
+          <t>images/judgment-05-Y1Dd_ASy9tc--1x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B152" s="11" t="inlineStr">
@@ -4866,7 +4866,7 @@
       </c>
       <c r="D152" s="11" t="inlineStr">
         <is>
-          <t>86.4 KB</t>
+          <t>122.0 KB</t>
         </is>
       </c>
       <c r="E152" s="12" t="inlineStr">
@@ -4878,7 +4878,7 @@
     <row r="153" ht="16" customHeight="1">
       <c r="A153" s="9" t="inlineStr">
         <is>
-          <t>images/signal-03-nwNjeZ0WA6w--16x9-textsafe.jpg</t>
+          <t>images/judgment-05-Y1Dd_ASy9tc--1x1.jpg</t>
         </is>
       </c>
       <c r="B153" s="9" t="inlineStr">
@@ -4893,7 +4893,7 @@
       </c>
       <c r="D153" s="9" t="inlineStr">
         <is>
-          <t>45.4 KB</t>
+          <t>159.9 KB</t>
         </is>
       </c>
       <c r="E153" s="10" t="inlineStr">
@@ -4905,7 +4905,7 @@
     <row r="154" ht="16" customHeight="1">
       <c r="A154" s="11" t="inlineStr">
         <is>
-          <t>images/signal-03-nwNjeZ0WA6w--16x9.jpg</t>
+          <t>images/judgment-05-Y1Dd_ASy9tc--2x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B154" s="11" t="inlineStr">
@@ -4920,7 +4920,7 @@
       </c>
       <c r="D154" s="11" t="inlineStr">
         <is>
-          <t>62.1 KB</t>
+          <t>166.3 KB</t>
         </is>
       </c>
       <c r="E154" s="12" t="inlineStr">
@@ -4932,7 +4932,7 @@
     <row r="155" ht="16" customHeight="1">
       <c r="A155" s="9" t="inlineStr">
         <is>
-          <t>images/signal-03-nwNjeZ0WA6w--1x1-textsafe.jpg</t>
+          <t>images/judgment-05-Y1Dd_ASy9tc--2x1.jpg</t>
         </is>
       </c>
       <c r="B155" s="9" t="inlineStr">
@@ -4947,7 +4947,7 @@
       </c>
       <c r="D155" s="9" t="inlineStr">
         <is>
-          <t>33.0 KB</t>
+          <t>217.0 KB</t>
         </is>
       </c>
       <c r="E155" s="10" t="inlineStr">
@@ -4959,7 +4959,7 @@
     <row r="156" ht="16" customHeight="1">
       <c r="A156" s="11" t="inlineStr">
         <is>
-          <t>images/signal-03-nwNjeZ0WA6w--1x1.jpg</t>
+          <t>images/judgment-05-Y1Dd_ASy9tc.jpg</t>
         </is>
       </c>
       <c r="B156" s="11" t="inlineStr">
@@ -4974,7 +4974,7 @@
       </c>
       <c r="D156" s="11" t="inlineStr">
         <is>
-          <t>45.4 KB</t>
+          <t>300.7 KB</t>
         </is>
       </c>
       <c r="E156" s="12" t="inlineStr">
@@ -4986,7 +4986,7 @@
     <row r="157" ht="16" customHeight="1">
       <c r="A157" s="9" t="inlineStr">
         <is>
-          <t>images/signal-03-nwNjeZ0WA6w--2x1-textsafe.jpg</t>
+          <t>images/signal-01-ux0tBq3xB60--16x9-textsafe.jpg</t>
         </is>
       </c>
       <c r="B157" s="9" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="D157" s="9" t="inlineStr">
         <is>
-          <t>41.6 KB</t>
+          <t>46.1 KB</t>
         </is>
       </c>
       <c r="E157" s="10" t="inlineStr">
@@ -5013,7 +5013,7 @@
     <row r="158" ht="16" customHeight="1">
       <c r="A158" s="11" t="inlineStr">
         <is>
-          <t>images/signal-03-nwNjeZ0WA6w--2x1.jpg</t>
+          <t>images/signal-01-ux0tBq3xB60--16x9.jpg</t>
         </is>
       </c>
       <c r="B158" s="11" t="inlineStr">
@@ -5028,7 +5028,7 @@
       </c>
       <c r="D158" s="11" t="inlineStr">
         <is>
-          <t>56.7 KB</t>
+          <t>64.6 KB</t>
         </is>
       </c>
       <c r="E158" s="12" t="inlineStr">
@@ -5040,7 +5040,7 @@
     <row r="159" ht="16" customHeight="1">
       <c r="A159" s="9" t="inlineStr">
         <is>
-          <t>images/signal-03-nwNjeZ0WA6w.jpg</t>
+          <t>images/signal-01-ux0tBq3xB60--1x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B159" s="9" t="inlineStr">
@@ -5055,7 +5055,7 @@
       </c>
       <c r="D159" s="9" t="inlineStr">
         <is>
-          <t>70.2 KB</t>
+          <t>38.3 KB</t>
         </is>
       </c>
       <c r="E159" s="10" t="inlineStr">
@@ -5067,7 +5067,7 @@
     <row r="160" ht="16" customHeight="1">
       <c r="A160" s="11" t="inlineStr">
         <is>
-          <t>images/signal-04-hT0nO6d2QVE--16x9-textsafe.jpg</t>
+          <t>images/signal-01-ux0tBq3xB60--1x1.jpg</t>
         </is>
       </c>
       <c r="B160" s="11" t="inlineStr">
@@ -5082,7 +5082,7 @@
       </c>
       <c r="D160" s="11" t="inlineStr">
         <is>
-          <t>93.4 KB</t>
+          <t>52.7 KB</t>
         </is>
       </c>
       <c r="E160" s="12" t="inlineStr">
@@ -5094,7 +5094,7 @@
     <row r="161" ht="16" customHeight="1">
       <c r="A161" s="9" t="inlineStr">
         <is>
-          <t>images/signal-04-hT0nO6d2QVE--16x9.jpg</t>
+          <t>images/signal-01-ux0tBq3xB60--2x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B161" s="9" t="inlineStr">
@@ -5109,7 +5109,7 @@
       </c>
       <c r="D161" s="9" t="inlineStr">
         <is>
-          <t>127.4 KB</t>
+          <t>40.9 KB</t>
         </is>
       </c>
       <c r="E161" s="10" t="inlineStr">
@@ -5121,7 +5121,7 @@
     <row r="162" ht="16" customHeight="1">
       <c r="A162" s="11" t="inlineStr">
         <is>
-          <t>images/signal-04-hT0nO6d2QVE--1x1-textsafe.jpg</t>
+          <t>images/signal-01-ux0tBq3xB60--2x1.jpg</t>
         </is>
       </c>
       <c r="B162" s="11" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="D162" s="11" t="inlineStr">
         <is>
-          <t>60.5 KB</t>
+          <t>57.4 KB</t>
         </is>
       </c>
       <c r="E162" s="12" t="inlineStr">
@@ -5148,7 +5148,7 @@
     <row r="163" ht="16" customHeight="1">
       <c r="A163" s="9" t="inlineStr">
         <is>
-          <t>images/signal-04-hT0nO6d2QVE--1x1.jpg</t>
+          <t>images/signal-01-ux0tBq3xB60.jpg</t>
         </is>
       </c>
       <c r="B163" s="9" t="inlineStr">
@@ -5163,7 +5163,7 @@
       </c>
       <c r="D163" s="9" t="inlineStr">
         <is>
-          <t>83.5 KB</t>
+          <t>103.1 KB</t>
         </is>
       </c>
       <c r="E163" s="10" t="inlineStr">
@@ -5175,7 +5175,7 @@
     <row r="164" ht="16" customHeight="1">
       <c r="A164" s="11" t="inlineStr">
         <is>
-          <t>images/signal-04-hT0nO6d2QVE--2x1-textsafe.jpg</t>
+          <t>images/signal-02-5RQyZZytm-Y--16x9-textsafe.jpg</t>
         </is>
       </c>
       <c r="B164" s="11" t="inlineStr">
@@ -5190,7 +5190,7 @@
       </c>
       <c r="D164" s="11" t="inlineStr">
         <is>
-          <t>84.3 KB</t>
+          <t>32.8 KB</t>
         </is>
       </c>
       <c r="E164" s="12" t="inlineStr">
@@ -5202,7 +5202,7 @@
     <row r="165" ht="16" customHeight="1">
       <c r="A165" s="9" t="inlineStr">
         <is>
-          <t>images/signal-04-hT0nO6d2QVE--2x1.jpg</t>
+          <t>images/signal-02-5RQyZZytm-Y--16x9.jpg</t>
         </is>
       </c>
       <c r="B165" s="9" t="inlineStr">
@@ -5217,7 +5217,7 @@
       </c>
       <c r="D165" s="9" t="inlineStr">
         <is>
-          <t>115.0 KB</t>
+          <t>53.9 KB</t>
         </is>
       </c>
       <c r="E165" s="10" t="inlineStr">
@@ -5229,7 +5229,7 @@
     <row r="166" ht="16" customHeight="1">
       <c r="A166" s="11" t="inlineStr">
         <is>
-          <t>images/signal-04-hT0nO6d2QVE.jpg</t>
+          <t>images/signal-02-5RQyZZytm-Y--1x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B166" s="11" t="inlineStr">
@@ -5244,7 +5244,7 @@
       </c>
       <c r="D166" s="11" t="inlineStr">
         <is>
-          <t>144.9 KB</t>
+          <t>24.6 KB</t>
         </is>
       </c>
       <c r="E166" s="12" t="inlineStr">
@@ -5256,303 +5256,762 @@
     <row r="167" ht="16" customHeight="1">
       <c r="A167" s="9" t="inlineStr">
         <is>
-          <t>logos/ai4comms-favicon-180.png</t>
+          <t>images/signal-02-5RQyZZytm-Y--1x1.jpg</t>
         </is>
       </c>
       <c r="B167" s="9" t="inlineStr">
         <is>
-          <t>logos</t>
+          <t>images</t>
         </is>
       </c>
       <c r="C167" s="9" t="inlineStr">
         <is>
-          <t>PNG</t>
+          <t>JPEG</t>
         </is>
       </c>
       <c r="D167" s="9" t="inlineStr">
         <is>
-          <t>4.0 KB</t>
+          <t>39.5 KB</t>
         </is>
       </c>
       <c r="E167" s="10" t="inlineStr">
         <is>
-          <t>Logo asset — ai4comms-favicon-180</t>
+          <t>Photography / imagery asset</t>
         </is>
       </c>
     </row>
     <row r="168" ht="16" customHeight="1">
       <c r="A168" s="11" t="inlineStr">
         <is>
-          <t>logos/ai4comms-favicon-192.png</t>
+          <t>images/signal-02-5RQyZZytm-Y--2x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B168" s="11" t="inlineStr">
         <is>
-          <t>logos</t>
+          <t>images</t>
         </is>
       </c>
       <c r="C168" s="11" t="inlineStr">
         <is>
-          <t>PNG</t>
+          <t>JPEG</t>
         </is>
       </c>
       <c r="D168" s="11" t="inlineStr">
         <is>
-          <t>4.2 KB</t>
+          <t>29.6 KB</t>
         </is>
       </c>
       <c r="E168" s="12" t="inlineStr">
         <is>
-          <t>Logo asset — ai4comms-favicon-192</t>
+          <t>Photography / imagery asset</t>
         </is>
       </c>
     </row>
     <row r="169" ht="16" customHeight="1">
       <c r="A169" s="9" t="inlineStr">
         <is>
-          <t>logos/ai4comms-logo-primary.png</t>
+          <t>images/signal-02-5RQyZZytm-Y--2x1.jpg</t>
         </is>
       </c>
       <c r="B169" s="9" t="inlineStr">
         <is>
-          <t>logos</t>
+          <t>images</t>
         </is>
       </c>
       <c r="C169" s="9" t="inlineStr">
         <is>
-          <t>PNG</t>
+          <t>JPEG</t>
         </is>
       </c>
       <c r="D169" s="9" t="inlineStr">
         <is>
-          <t>57.5 KB</t>
+          <t>48.3 KB</t>
         </is>
       </c>
       <c r="E169" s="10" t="inlineStr">
         <is>
-          <t>Logo asset — ai4comms-logo-primary</t>
+          <t>Photography / imagery asset</t>
         </is>
       </c>
     </row>
     <row r="170" ht="16" customHeight="1">
       <c r="A170" s="11" t="inlineStr">
         <is>
-          <t>logos/ai4comms-logo-primary.svg</t>
+          <t>images/signal-02-5RQyZZytm-Y.jpg</t>
         </is>
       </c>
       <c r="B170" s="11" t="inlineStr">
         <is>
-          <t>logos</t>
+          <t>images</t>
         </is>
       </c>
       <c r="C170" s="11" t="inlineStr">
         <is>
-          <t>SVG</t>
+          <t>JPEG</t>
         </is>
       </c>
       <c r="D170" s="11" t="inlineStr">
         <is>
-          <t>8.2 KB</t>
+          <t>86.4 KB</t>
         </is>
       </c>
       <c r="E170" s="12" t="inlineStr">
         <is>
-          <t>Logo asset — ai4comms-logo-primary</t>
+          <t>Photography / imagery asset</t>
         </is>
       </c>
     </row>
     <row r="171" ht="16" customHeight="1">
       <c r="A171" s="9" t="inlineStr">
         <is>
-          <t>profile.json</t>
+          <t>images/signal-03-nwNjeZ0WA6w--16x9-textsafe.jpg</t>
         </is>
       </c>
       <c r="B171" s="9" t="inlineStr">
         <is>
-          <t>root</t>
+          <t>images</t>
         </is>
       </c>
       <c r="C171" s="9" t="inlineStr">
         <is>
-          <t>JSON</t>
+          <t>JPEG</t>
         </is>
       </c>
       <c r="D171" s="9" t="inlineStr">
         <is>
-          <t>3.7 KB</t>
+          <t>45.4 KB</t>
         </is>
       </c>
       <c r="E171" s="10" t="inlineStr">
         <is>
-          <t>Company profile — description, services, legal identity</t>
+          <t>Photography / imagery asset</t>
         </is>
       </c>
     </row>
     <row r="172" ht="16" customHeight="1">
       <c r="A172" s="11" t="inlineStr">
         <is>
-          <t>proposals/.gitkeep</t>
+          <t>images/signal-03-nwNjeZ0WA6w--16x9.jpg</t>
         </is>
       </c>
       <c r="B172" s="11" t="inlineStr">
         <is>
-          <t>proposals</t>
+          <t>images</t>
         </is>
       </c>
       <c r="C172" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>JPEG</t>
         </is>
       </c>
       <c r="D172" s="11" t="inlineStr">
         <is>
-          <t>0.0 KB</t>
+          <t>62.1 KB</t>
         </is>
       </c>
       <c r="E172" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Photography / imagery asset</t>
         </is>
       </c>
     </row>
     <row r="173" ht="16" customHeight="1">
       <c r="A173" s="9" t="inlineStr">
         <is>
-          <t>templates/docx/default.docx</t>
+          <t>images/signal-03-nwNjeZ0WA6w--1x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B173" s="9" t="inlineStr">
         <is>
-          <t>templates</t>
+          <t>images</t>
         </is>
       </c>
       <c r="C173" s="9" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>JPEG</t>
         </is>
       </c>
       <c r="D173" s="9" t="inlineStr">
         <is>
-          <t>151.0 KB</t>
+          <t>33.0 KB</t>
         </is>
       </c>
       <c r="E173" s="10" t="inlineStr">
         <is>
-          <t>Branded Word styles template</t>
+          <t>Photography / imagery asset</t>
         </is>
       </c>
     </row>
     <row r="174" ht="16" customHeight="1">
       <c r="A174" s="11" t="inlineStr">
         <is>
-          <t>templates/docx/letterhead.docx</t>
+          <t>images/signal-03-nwNjeZ0WA6w--1x1.jpg</t>
         </is>
       </c>
       <c r="B174" s="11" t="inlineStr">
         <is>
-          <t>templates</t>
+          <t>images</t>
         </is>
       </c>
       <c r="C174" s="11" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>JPEG</t>
         </is>
       </c>
       <c r="D174" s="11" t="inlineStr">
         <is>
-          <t>32.4 KB</t>
+          <t>45.4 KB</t>
         </is>
       </c>
       <c r="E174" s="12" t="inlineStr">
         <is>
-          <t>Branded Word styles template</t>
+          <t>Photography / imagery asset</t>
         </is>
       </c>
     </row>
     <row r="175" ht="16" customHeight="1">
       <c r="A175" s="9" t="inlineStr">
         <is>
-          <t>templates/html/business-cards.html</t>
+          <t>images/signal-03-nwNjeZ0WA6w--2x1-textsafe.jpg</t>
         </is>
       </c>
       <c r="B175" s="9" t="inlineStr">
         <is>
-          <t>templates</t>
+          <t>images</t>
         </is>
       </c>
       <c r="C175" s="9" t="inlineStr">
         <is>
-          <t>HTML</t>
+          <t>JPEG</t>
         </is>
       </c>
       <c r="D175" s="9" t="inlineStr">
         <is>
-          <t>12.7 KB</t>
+          <t>41.6 KB</t>
         </is>
       </c>
       <c r="E175" s="10" t="inlineStr">
         <is>
-          <t>Branded HTML template</t>
+          <t>Photography / imagery asset</t>
         </is>
       </c>
     </row>
     <row r="176" ht="16" customHeight="1">
       <c r="A176" s="11" t="inlineStr">
         <is>
-          <t>templates/html/email-signature.html</t>
+          <t>images/signal-03-nwNjeZ0WA6w--2x1.jpg</t>
         </is>
       </c>
       <c r="B176" s="11" t="inlineStr">
         <is>
-          <t>templates</t>
+          <t>images</t>
         </is>
       </c>
       <c r="C176" s="11" t="inlineStr">
         <is>
-          <t>HTML</t>
+          <t>JPEG</t>
         </is>
       </c>
       <c r="D176" s="11" t="inlineStr">
         <is>
-          <t>9.3 KB</t>
+          <t>56.7 KB</t>
         </is>
       </c>
       <c r="E176" s="12" t="inlineStr">
         <is>
-          <t>Branded HTML template</t>
+          <t>Photography / imagery asset</t>
         </is>
       </c>
     </row>
     <row r="177" ht="16" customHeight="1">
       <c r="A177" s="9" t="inlineStr">
         <is>
+          <t>images/signal-03-nwNjeZ0WA6w.jpg</t>
+        </is>
+      </c>
+      <c r="B177" s="9" t="inlineStr">
+        <is>
+          <t>images</t>
+        </is>
+      </c>
+      <c r="C177" s="9" t="inlineStr">
+        <is>
+          <t>JPEG</t>
+        </is>
+      </c>
+      <c r="D177" s="9" t="inlineStr">
+        <is>
+          <t>70.2 KB</t>
+        </is>
+      </c>
+      <c r="E177" s="10" t="inlineStr">
+        <is>
+          <t>Photography / imagery asset</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" ht="16" customHeight="1">
+      <c r="A178" s="11" t="inlineStr">
+        <is>
+          <t>images/signal-04-hT0nO6d2QVE--16x9-textsafe.jpg</t>
+        </is>
+      </c>
+      <c r="B178" s="11" t="inlineStr">
+        <is>
+          <t>images</t>
+        </is>
+      </c>
+      <c r="C178" s="11" t="inlineStr">
+        <is>
+          <t>JPEG</t>
+        </is>
+      </c>
+      <c r="D178" s="11" t="inlineStr">
+        <is>
+          <t>93.4 KB</t>
+        </is>
+      </c>
+      <c r="E178" s="12" t="inlineStr">
+        <is>
+          <t>Photography / imagery asset</t>
+        </is>
+      </c>
+    </row>
+    <row r="179" ht="16" customHeight="1">
+      <c r="A179" s="9" t="inlineStr">
+        <is>
+          <t>images/signal-04-hT0nO6d2QVE--16x9.jpg</t>
+        </is>
+      </c>
+      <c r="B179" s="9" t="inlineStr">
+        <is>
+          <t>images</t>
+        </is>
+      </c>
+      <c r="C179" s="9" t="inlineStr">
+        <is>
+          <t>JPEG</t>
+        </is>
+      </c>
+      <c r="D179" s="9" t="inlineStr">
+        <is>
+          <t>127.4 KB</t>
+        </is>
+      </c>
+      <c r="E179" s="10" t="inlineStr">
+        <is>
+          <t>Photography / imagery asset</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="16" customHeight="1">
+      <c r="A180" s="11" t="inlineStr">
+        <is>
+          <t>images/signal-04-hT0nO6d2QVE--1x1-textsafe.jpg</t>
+        </is>
+      </c>
+      <c r="B180" s="11" t="inlineStr">
+        <is>
+          <t>images</t>
+        </is>
+      </c>
+      <c r="C180" s="11" t="inlineStr">
+        <is>
+          <t>JPEG</t>
+        </is>
+      </c>
+      <c r="D180" s="11" t="inlineStr">
+        <is>
+          <t>60.5 KB</t>
+        </is>
+      </c>
+      <c r="E180" s="12" t="inlineStr">
+        <is>
+          <t>Photography / imagery asset</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" ht="16" customHeight="1">
+      <c r="A181" s="9" t="inlineStr">
+        <is>
+          <t>images/signal-04-hT0nO6d2QVE--1x1.jpg</t>
+        </is>
+      </c>
+      <c r="B181" s="9" t="inlineStr">
+        <is>
+          <t>images</t>
+        </is>
+      </c>
+      <c r="C181" s="9" t="inlineStr">
+        <is>
+          <t>JPEG</t>
+        </is>
+      </c>
+      <c r="D181" s="9" t="inlineStr">
+        <is>
+          <t>83.5 KB</t>
+        </is>
+      </c>
+      <c r="E181" s="10" t="inlineStr">
+        <is>
+          <t>Photography / imagery asset</t>
+        </is>
+      </c>
+    </row>
+    <row r="182" ht="16" customHeight="1">
+      <c r="A182" s="11" t="inlineStr">
+        <is>
+          <t>images/signal-04-hT0nO6d2QVE--2x1-textsafe.jpg</t>
+        </is>
+      </c>
+      <c r="B182" s="11" t="inlineStr">
+        <is>
+          <t>images</t>
+        </is>
+      </c>
+      <c r="C182" s="11" t="inlineStr">
+        <is>
+          <t>JPEG</t>
+        </is>
+      </c>
+      <c r="D182" s="11" t="inlineStr">
+        <is>
+          <t>84.3 KB</t>
+        </is>
+      </c>
+      <c r="E182" s="12" t="inlineStr">
+        <is>
+          <t>Photography / imagery asset</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" ht="16" customHeight="1">
+      <c r="A183" s="9" t="inlineStr">
+        <is>
+          <t>images/signal-04-hT0nO6d2QVE--2x1.jpg</t>
+        </is>
+      </c>
+      <c r="B183" s="9" t="inlineStr">
+        <is>
+          <t>images</t>
+        </is>
+      </c>
+      <c r="C183" s="9" t="inlineStr">
+        <is>
+          <t>JPEG</t>
+        </is>
+      </c>
+      <c r="D183" s="9" t="inlineStr">
+        <is>
+          <t>115.0 KB</t>
+        </is>
+      </c>
+      <c r="E183" s="10" t="inlineStr">
+        <is>
+          <t>Photography / imagery asset</t>
+        </is>
+      </c>
+    </row>
+    <row r="184" ht="16" customHeight="1">
+      <c r="A184" s="11" t="inlineStr">
+        <is>
+          <t>images/signal-04-hT0nO6d2QVE.jpg</t>
+        </is>
+      </c>
+      <c r="B184" s="11" t="inlineStr">
+        <is>
+          <t>images</t>
+        </is>
+      </c>
+      <c r="C184" s="11" t="inlineStr">
+        <is>
+          <t>JPEG</t>
+        </is>
+      </c>
+      <c r="D184" s="11" t="inlineStr">
+        <is>
+          <t>144.9 KB</t>
+        </is>
+      </c>
+      <c r="E184" s="12" t="inlineStr">
+        <is>
+          <t>Photography / imagery asset</t>
+        </is>
+      </c>
+    </row>
+    <row r="185" ht="16" customHeight="1">
+      <c r="A185" s="9" t="inlineStr">
+        <is>
+          <t>logos/ai4comms-favicon-180.png</t>
+        </is>
+      </c>
+      <c r="B185" s="9" t="inlineStr">
+        <is>
+          <t>logos</t>
+        </is>
+      </c>
+      <c r="C185" s="9" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="D185" s="9" t="inlineStr">
+        <is>
+          <t>4.0 KB</t>
+        </is>
+      </c>
+      <c r="E185" s="10" t="inlineStr">
+        <is>
+          <t>Logo asset — ai4comms-favicon-180</t>
+        </is>
+      </c>
+    </row>
+    <row r="186" ht="16" customHeight="1">
+      <c r="A186" s="11" t="inlineStr">
+        <is>
+          <t>logos/ai4comms-favicon-192.png</t>
+        </is>
+      </c>
+      <c r="B186" s="11" t="inlineStr">
+        <is>
+          <t>logos</t>
+        </is>
+      </c>
+      <c r="C186" s="11" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="D186" s="11" t="inlineStr">
+        <is>
+          <t>4.2 KB</t>
+        </is>
+      </c>
+      <c r="E186" s="12" t="inlineStr">
+        <is>
+          <t>Logo asset — ai4comms-favicon-192</t>
+        </is>
+      </c>
+    </row>
+    <row r="187" ht="16" customHeight="1">
+      <c r="A187" s="9" t="inlineStr">
+        <is>
+          <t>logos/ai4comms-logo-primary.png</t>
+        </is>
+      </c>
+      <c r="B187" s="9" t="inlineStr">
+        <is>
+          <t>logos</t>
+        </is>
+      </c>
+      <c r="C187" s="9" t="inlineStr">
+        <is>
+          <t>PNG</t>
+        </is>
+      </c>
+      <c r="D187" s="9" t="inlineStr">
+        <is>
+          <t>57.5 KB</t>
+        </is>
+      </c>
+      <c r="E187" s="10" t="inlineStr">
+        <is>
+          <t>Logo asset — ai4comms-logo-primary</t>
+        </is>
+      </c>
+    </row>
+    <row r="188" ht="16" customHeight="1">
+      <c r="A188" s="11" t="inlineStr">
+        <is>
+          <t>logos/ai4comms-logo-primary.svg</t>
+        </is>
+      </c>
+      <c r="B188" s="11" t="inlineStr">
+        <is>
+          <t>logos</t>
+        </is>
+      </c>
+      <c r="C188" s="11" t="inlineStr">
+        <is>
+          <t>SVG</t>
+        </is>
+      </c>
+      <c r="D188" s="11" t="inlineStr">
+        <is>
+          <t>8.2 KB</t>
+        </is>
+      </c>
+      <c r="E188" s="12" t="inlineStr">
+        <is>
+          <t>Logo asset — ai4comms-logo-primary</t>
+        </is>
+      </c>
+    </row>
+    <row r="189" ht="16" customHeight="1">
+      <c r="A189" s="9" t="inlineStr">
+        <is>
+          <t>profile.json</t>
+        </is>
+      </c>
+      <c r="B189" s="9" t="inlineStr">
+        <is>
+          <t>root</t>
+        </is>
+      </c>
+      <c r="C189" s="9" t="inlineStr">
+        <is>
+          <t>JSON</t>
+        </is>
+      </c>
+      <c r="D189" s="9" t="inlineStr">
+        <is>
+          <t>3.7 KB</t>
+        </is>
+      </c>
+      <c r="E189" s="10" t="inlineStr">
+        <is>
+          <t>Company profile — description, services, legal identity</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" ht="16" customHeight="1">
+      <c r="A190" s="11" t="inlineStr">
+        <is>
+          <t>proposals/.gitkeep</t>
+        </is>
+      </c>
+      <c r="B190" s="11" t="inlineStr">
+        <is>
+          <t>proposals</t>
+        </is>
+      </c>
+      <c r="C190" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D190" s="11" t="inlineStr">
+        <is>
+          <t>0.0 KB</t>
+        </is>
+      </c>
+      <c r="E190" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="16" customHeight="1">
+      <c r="A191" s="9" t="inlineStr">
+        <is>
+          <t>templates/docx/default.docx</t>
+        </is>
+      </c>
+      <c r="B191" s="9" t="inlineStr">
+        <is>
+          <t>templates</t>
+        </is>
+      </c>
+      <c r="C191" s="9" t="inlineStr">
+        <is>
+          <t>DOCX</t>
+        </is>
+      </c>
+      <c r="D191" s="9" t="inlineStr">
+        <is>
+          <t>151.0 KB</t>
+        </is>
+      </c>
+      <c r="E191" s="10" t="inlineStr">
+        <is>
+          <t>Branded Word styles template</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" ht="16" customHeight="1">
+      <c r="A192" s="11" t="inlineStr">
+        <is>
+          <t>templates/docx/letterhead.docx</t>
+        </is>
+      </c>
+      <c r="B192" s="11" t="inlineStr">
+        <is>
+          <t>templates</t>
+        </is>
+      </c>
+      <c r="C192" s="11" t="inlineStr">
+        <is>
+          <t>DOCX</t>
+        </is>
+      </c>
+      <c r="D192" s="11" t="inlineStr">
+        <is>
+          <t>32.4 KB</t>
+        </is>
+      </c>
+      <c r="E192" s="12" t="inlineStr">
+        <is>
+          <t>Branded Word styles template</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" ht="16" customHeight="1">
+      <c r="A193" s="9" t="inlineStr">
+        <is>
+          <t>templates/html/email-signature.html</t>
+        </is>
+      </c>
+      <c r="B193" s="9" t="inlineStr">
+        <is>
+          <t>templates</t>
+        </is>
+      </c>
+      <c r="C193" s="9" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="D193" s="9" t="inlineStr">
+        <is>
+          <t>9.3 KB</t>
+        </is>
+      </c>
+      <c r="E193" s="10" t="inlineStr">
+        <is>
+          <t>Branded HTML template</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" ht="16" customHeight="1">
+      <c r="A194" s="11" t="inlineStr">
+        <is>
           <t>tokens.css</t>
         </is>
       </c>
-      <c r="B177" s="9" t="inlineStr">
+      <c r="B194" s="11" t="inlineStr">
         <is>
           <t>root</t>
         </is>
       </c>
-      <c r="C177" s="9" t="inlineStr">
+      <c r="C194" s="11" t="inlineStr">
         <is>
           <t>CSS</t>
         </is>
       </c>
-      <c r="D177" s="9" t="inlineStr">
+      <c r="D194" s="11" t="inlineStr">
         <is>
           <t>7.8 KB</t>
         </is>
       </c>
-      <c r="E177" s="10" t="inlineStr">
+      <c r="E194" s="12" t="inlineStr">
         <is>
           <t>CSS design tokens mapping brand colors to CSS variables</t>
         </is>
       </c>
     </row>
-    <row r="178" ht="8" customHeight="1"/>
-    <row r="179">
-      <c r="A179" s="7" t="inlineStr">
+    <row r="195" ht="8" customHeight="1"/>
+    <row r="196">
+      <c r="A196" s="7" t="inlineStr">
         <is>
           <t>AI4comms  ·  Confidential — Not for distribution</t>
         </is>
@@ -5561,7 +6020,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A179:F179"/>
+    <mergeCell ref="A196:F196"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6188,7 +6647,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>background</t>
+          <t>primary</t>
         </is>
       </c>
     </row>
@@ -6212,7 +6671,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>white</t>
+          <t>primary</t>
         </is>
       </c>
     </row>

</xml_diff>